<commit_message>
Projections through August 13
Sixty-six changes: twenty-eight updated, twenty-one reconciled, two ruled
out, and seven looked at and left alone.
</commit_message>
<xml_diff>
--- a/data/projections.xlsx
+++ b/data/projections.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QB" sheetId="1" r:id="Rca03c9baec8e4f10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="2" r:id="R0035250046574680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WR" sheetId="3" r:id="R21950035cf3f4e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TE" sheetId="4" r:id="Rf173777255d643a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Update" sheetId="5" r:id="R64b6e7b8e87a4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QB" sheetId="1" r:id="Rae9978c93ab44872"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="2" r:id="R30987d1a9b8749dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WR" sheetId="3" r:id="R1afdb2d94fde486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TE" sheetId="4" r:id="R67e4950c854f4464"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Update" sheetId="5" r:id="Rea8a9344b9f94322"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -43,8 +43,13 @@
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -86,6 +91,16 @@
         <x:fgColor rgb="FFFFF7E6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F2937"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="18">
     <x:border/>
@@ -110,7 +125,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="95">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -272,6 +287,58 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2369,7 +2436,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7611a4b7340343c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec580ede0e2c4ed1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3763,43 +3830,43 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B32" s="20" t="str">
-        <x:v>Chuba Hubbard</x:v>
+        <x:v>Rico Dowdle</x:v>
       </x:c>
       <x:c r="C32" s="16" t="str">
-        <x:v>CAR</x:v>
+        <x:v>PIT</x:v>
       </x:c>
       <x:c r="D32" s="17" t="n">
-        <x:v>38.4</x:v>
+        <x:v>37.7</x:v>
       </x:c>
       <x:c r="E32" s="17" t="n">
-        <x:v>29.4</x:v>
+        <x:v>27.8</x:v>
       </x:c>
       <x:c r="F32" s="17" t="n">
-        <x:v>201.6</x:v>
+        <x:v>193.2</x:v>
       </x:c>
       <x:c r="G32" s="17" t="n">
-        <x:v>1.37</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="H32" s="17" t="n">
-        <x:v>180</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="I32" s="17" t="n">
-        <x:v>738</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="J32" s="17" t="n">
-        <x:v>4.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K32" s="17" t="n">
-        <x:v>1.3</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="L32" s="17" t="n">
         <x:v>156</x:v>
       </x:c>
       <x:c r="M32" s="17" t="n">
-        <x:v>141.3</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="N32" s="26" t="n">
-        <x:v>126.6</x:v>
+        <x:v>128.1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -3807,43 +3874,43 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B33" s="20" t="str">
-        <x:v>Rico Dowdle</x:v>
+        <x:v>Rhamondre Stevenson</x:v>
       </x:c>
       <x:c r="C33" s="16" t="str">
-        <x:v>PIT</x:v>
+        <x:v>NE</x:v>
       </x:c>
       <x:c r="D33" s="17" t="n">
-        <x:v>37.7</x:v>
+        <x:v>38.5</x:v>
       </x:c>
       <x:c r="E33" s="17" t="n">
-        <x:v>27.8</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="F33" s="17" t="n">
-        <x:v>193.2</x:v>
+        <x:v>267.2</x:v>
       </x:c>
       <x:c r="G33" s="17" t="n">
-        <x:v>0.8</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="H33" s="17" t="n">
-        <x:v>175</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="I33" s="17" t="n">
-        <x:v>760</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="J33" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="K33" s="17" t="n">
-        <x:v>0.9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L33" s="17" t="n">
-        <x:v>156</x:v>
+        <x:v>152.8</x:v>
       </x:c>
       <x:c r="M33" s="17" t="n">
-        <x:v>142</x:v>
+        <x:v>137.3</x:v>
       </x:c>
       <x:c r="N33" s="26" t="n">
-        <x:v>128.1</x:v>
+        <x:v>121.8</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
@@ -3851,43 +3918,43 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B34" s="20" t="str">
-        <x:v>Rhamondre Stevenson</x:v>
+        <x:v>Kenny Gainwell</x:v>
       </x:c>
       <x:c r="C34" s="16" t="str">
-        <x:v>NE</x:v>
+        <x:v>TB</x:v>
       </x:c>
       <x:c r="D34" s="17" t="n">
-        <x:v>38.5</x:v>
+        <x:v>55.6</x:v>
       </x:c>
       <x:c r="E34" s="17" t="n">
-        <x:v>31</x:v>
+        <x:v>41.9</x:v>
       </x:c>
       <x:c r="F34" s="17" t="n">
-        <x:v>267.2</x:v>
+        <x:v>294.1</x:v>
       </x:c>
       <x:c r="G34" s="17" t="n">
-        <x:v>1.1</x:v>
+        <x:v>1.6</x:v>
       </x:c>
       <x:c r="H34" s="17" t="n">
-        <x:v>145</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="I34" s="17" t="n">
-        <x:v>625</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="J34" s="17" t="n">
-        <x:v>5</x:v>
+        <x:v>3.7</x:v>
       </x:c>
       <x:c r="K34" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="L34" s="17" t="n">
-        <x:v>152.8</x:v>
+        <x:v>151.3</x:v>
       </x:c>
       <x:c r="M34" s="17" t="n">
-        <x:v>137.3</x:v>
+        <x:v>130.4</x:v>
       </x:c>
       <x:c r="N34" s="26" t="n">
-        <x:v>121.8</x:v>
+        <x:v>109.4</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
@@ -3895,43 +3962,43 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B35" s="20" t="str">
-        <x:v>Kenny Gainwell</x:v>
+        <x:v>Kyle Monangai</x:v>
       </x:c>
       <x:c r="C35" s="16" t="str">
-        <x:v>TB</x:v>
+        <x:v>CHI</x:v>
       </x:c>
       <x:c r="D35" s="17" t="n">
-        <x:v>55.6</x:v>
+        <x:v>29.9</x:v>
       </x:c>
       <x:c r="E35" s="17" t="n">
-        <x:v>41.9</x:v>
+        <x:v>21.4</x:v>
       </x:c>
       <x:c r="F35" s="17" t="n">
-        <x:v>294.1</x:v>
+        <x:v>173.1</x:v>
       </x:c>
       <x:c r="G35" s="17" t="n">
-        <x:v>1.6</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H35" s="17" t="n">
-        <x:v>115</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="I35" s="17" t="n">
-        <x:v>500</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="J35" s="17" t="n">
-        <x:v>3.7</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="K35" s="17" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="L35" s="17" t="n">
-        <x:v>151.3</x:v>
+        <x:v>146.6</x:v>
       </x:c>
       <x:c r="M35" s="17" t="n">
-        <x:v>130.4</x:v>
+        <x:v>135.9</x:v>
       </x:c>
       <x:c r="N35" s="26" t="n">
-        <x:v>109.4</x:v>
+        <x:v>125.3</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -3939,43 +4006,43 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B36" s="20" t="str">
-        <x:v>Kyle Monangai</x:v>
+        <x:v>Chuba Hubbard</x:v>
       </x:c>
       <x:c r="C36" s="16" t="str">
-        <x:v>CHI</x:v>
+        <x:v>CAR</x:v>
       </x:c>
       <x:c r="D36" s="17" t="n">
-        <x:v>29.9</x:v>
+        <x:v>35.4</x:v>
       </x:c>
       <x:c r="E36" s="17" t="n">
-        <x:v>21.4</x:v>
+        <x:v>27.1</x:v>
       </x:c>
       <x:c r="F36" s="17" t="n">
-        <x:v>173.1</x:v>
+        <x:v>185.9</x:v>
       </x:c>
       <x:c r="G36" s="17" t="n">
-        <x:v>0.4</x:v>
+        <x:v>1.26</x:v>
       </x:c>
       <x:c r="H36" s="17" t="n">
-        <x:v>180</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="I36" s="17" t="n">
-        <x:v>770</x:v>
+        <x:v>688.8</x:v>
       </x:c>
       <x:c r="J36" s="17" t="n">
-        <x:v>5</x:v>
+        <x:v>4.2</x:v>
       </x:c>
       <x:c r="K36" s="17" t="n">
-        <x:v>0.7</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L36" s="17" t="n">
-        <x:v>146.6</x:v>
+        <x:v>144.9</x:v>
       </x:c>
       <x:c r="M36" s="17" t="n">
-        <x:v>135.9</x:v>
+        <x:v>131.4</x:v>
       </x:c>
       <x:c r="N36" s="26" t="n">
-        <x:v>125.3</x:v>
+        <x:v>117.8</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -3983,43 +4050,43 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
-        <x:v>Aaron Jones Sr.</x:v>
+        <x:v>Jonathon Brooks</x:v>
       </x:c>
       <x:c r="C37" s="16" t="str">
-        <x:v>MIN</x:v>
+        <x:v>CAR</x:v>
       </x:c>
       <x:c r="D37" s="17" t="n">
-        <x:v>46.1</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E37" s="17" t="n">
-        <x:v>35</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F37" s="17" t="n">
-        <x:v>255.3</x:v>
+        <x:v>208.2</x:v>
       </x:c>
       <x:c r="G37" s="17" t="n">
-        <x:v>1.4</x:v>
+        <x:v>0.99</x:v>
       </x:c>
       <x:c r="H37" s="17" t="n">
-        <x:v>130</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I37" s="17" t="n">
-        <x:v>560</x:v>
+        <x:v>649.2</x:v>
       </x:c>
       <x:c r="J37" s="17" t="n">
-        <x:v>3.2</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="K37" s="17" t="n">
-        <x:v>1.2</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="L37" s="17" t="n">
-        <x:v>142</x:v>
+        <x:v>142.7</x:v>
       </x:c>
       <x:c r="M37" s="17" t="n">
-        <x:v>124.5</x:v>
+        <x:v>129.2</x:v>
       </x:c>
       <x:c r="N37" s="26" t="n">
-        <x:v>107</x:v>
+        <x:v>115.7</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
@@ -4027,43 +4094,43 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
-        <x:v>RJ Harvey</x:v>
+        <x:v>Aaron Jones Sr.</x:v>
       </x:c>
       <x:c r="C38" s="16" t="str">
-        <x:v>DEN</x:v>
+        <x:v>MIN</x:v>
       </x:c>
       <x:c r="D38" s="17" t="n">
-        <x:v>45.2</x:v>
+        <x:v>46.1</x:v>
       </x:c>
       <x:c r="E38" s="17" t="n">
-        <x:v>32.9</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F38" s="17" t="n">
-        <x:v>242.1</x:v>
+        <x:v>255.3</x:v>
       </x:c>
       <x:c r="G38" s="17" t="n">
-        <x:v>2.5</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="H38" s="17" t="n">
-        <x:v>108.7</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="I38" s="17" t="n">
-        <x:v>409.6</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="J38" s="17" t="n">
-        <x:v>3.9</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="K38" s="17" t="n">
-        <x:v>0.6</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L38" s="17" t="n">
-        <x:v>135.1</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="M38" s="17" t="n">
-        <x:v>118.7</x:v>
+        <x:v>124.5</x:v>
       </x:c>
       <x:c r="N38" s="26" t="n">
-        <x:v>102.2</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -4071,43 +4138,43 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B39" s="20" t="str">
-        <x:v>J.K. Dobbins</x:v>
+        <x:v>RJ Harvey</x:v>
       </x:c>
       <x:c r="C39" s="16" t="str">
         <x:v>DEN</x:v>
       </x:c>
       <x:c r="D39" s="17" t="n">
-        <x:v>19.5</x:v>
+        <x:v>45.2</x:v>
       </x:c>
       <x:c r="E39" s="17" t="n">
-        <x:v>14.3</x:v>
+        <x:v>32.9</x:v>
       </x:c>
       <x:c r="F39" s="17" t="n">
-        <x:v>76.3</x:v>
+        <x:v>242.1</x:v>
       </x:c>
       <x:c r="G39" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H39" s="17" t="n">
-        <x:v>175</x:v>
+        <x:v>108.7</x:v>
       </x:c>
       <x:c r="I39" s="17" t="n">
-        <x:v>800</x:v>
+        <x:v>409.6</x:v>
       </x:c>
       <x:c r="J39" s="17" t="n">
-        <x:v>5.5</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="K39" s="17" t="n">
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="L39" s="17" t="n">
-        <x:v>134.9</x:v>
+        <x:v>135.1</x:v>
       </x:c>
       <x:c r="M39" s="17" t="n">
-        <x:v>127.7</x:v>
+        <x:v>118.7</x:v>
       </x:c>
       <x:c r="N39" s="26" t="n">
-        <x:v>120.6</x:v>
+        <x:v>102.2</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
@@ -4115,43 +4182,43 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B40" s="20" t="str">
-        <x:v>Blake Corum</x:v>
+        <x:v>J.K. Dobbins</x:v>
       </x:c>
       <x:c r="C40" s="16" t="str">
-        <x:v>LAR</x:v>
+        <x:v>DEN</x:v>
       </x:c>
       <x:c r="D40" s="17" t="n">
-        <x:v>16.3</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="E40" s="17" t="n">
-        <x:v>11.8</x:v>
+        <x:v>14.3</x:v>
       </x:c>
       <x:c r="F40" s="17" t="n">
-        <x:v>81.1</x:v>
+        <x:v>76.3</x:v>
       </x:c>
       <x:c r="G40" s="17" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H40" s="17" t="n">
-        <x:v>165</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="I40" s="17" t="n">
-        <x:v>790</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="J40" s="17" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="K40" s="17" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="L40" s="17" t="n">
-        <x:v>134</x:v>
+        <x:v>134.9</x:v>
       </x:c>
       <x:c r="M40" s="17" t="n">
-        <x:v>128.1</x:v>
+        <x:v>127.7</x:v>
       </x:c>
       <x:c r="N40" s="26" t="n">
-        <x:v>122.2</x:v>
+        <x:v>120.6</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -4159,43 +4226,43 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B41" s="20" t="str">
-        <x:v>Jonathon Brooks</x:v>
+        <x:v>Blake Corum</x:v>
       </x:c>
       <x:c r="C41" s="16" t="str">
-        <x:v>CAR</x:v>
+        <x:v>LAR</x:v>
       </x:c>
       <x:c r="D41" s="17" t="n">
-        <x:v>34</x:v>
+        <x:v>16.3</x:v>
       </x:c>
       <x:c r="E41" s="17" t="n">
-        <x:v>24.7</x:v>
+        <x:v>11.8</x:v>
       </x:c>
       <x:c r="F41" s="17" t="n">
-        <x:v>192.5</x:v>
+        <x:v>81.1</x:v>
       </x:c>
       <x:c r="G41" s="17" t="n">
-        <x:v>0.88</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="H41" s="17" t="n">
-        <x:v>145</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="I41" s="17" t="n">
-        <x:v>600</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="J41" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="K41" s="17" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="L41" s="17" t="n">
-        <x:v>131.6</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="M41" s="17" t="n">
-        <x:v>119.3</x:v>
+        <x:v>128.1</x:v>
       </x:c>
       <x:c r="N41" s="26" t="n">
-        <x:v>106.9</x:v>
+        <x:v>122.2</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
@@ -9568,7 +9635,7 @@
     </x:row>
     <x:row r="164" ht="15" hidden="0" customHeight="1">
       <x:c r="A164" s="25" t="n">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B164" s="20" t="str">
         <x:v>Zavier Scott</x:v>
@@ -9612,7 +9679,7 @@
     </x:row>
     <x:row r="165" ht="15" hidden="0" customHeight="1">
       <x:c r="A165" s="25" t="n">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B165" s="20" t="str">
         <x:v>Dylan Laube</x:v>
@@ -9656,7 +9723,7 @@
     </x:row>
     <x:row r="166" ht="15" hidden="0" customHeight="1">
       <x:c r="A166" s="25" t="n">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B166" s="20" t="str">
         <x:v>Dare Ogunbowale</x:v>
@@ -9700,7 +9767,7 @@
     </x:row>
     <x:row r="167" ht="15" hidden="0" customHeight="1">
       <x:c r="A167" s="25" t="n">
-        <x:v>167</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B167" s="20" t="str">
         <x:v>Bam Knight</x:v>
@@ -9744,7 +9811,7 @@
     </x:row>
     <x:row r="168" ht="15" hidden="0" customHeight="1">
       <x:c r="A168" s="25" t="n">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B168" s="20" t="str">
         <x:v>Corey Kiner</x:v>
@@ -9788,7 +9855,7 @@
     </x:row>
     <x:row r="169" ht="15" hidden="0" customHeight="1">
       <x:c r="A169" s="27" t="n">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B169" s="28" t="str">
         <x:v>Trey Benson</x:v>
@@ -9833,7 +9900,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f987317f7b64364"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0491a3bb7dd4407b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12371,43 +12438,43 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" s="20" t="str">
-        <x:v>Makai Lemon</x:v>
+        <x:v>KC Concepcion</x:v>
       </x:c>
       <x:c r="C58" s="16" t="str">
-        <x:v>PHI</x:v>
+        <x:v>CLE</x:v>
       </x:c>
       <x:c r="D58" s="17" t="n">
-        <x:v>74</x:v>
+        <x:v>74.4</x:v>
       </x:c>
       <x:c r="E58" s="17" t="n">
-        <x:v>44.4</x:v>
+        <x:v>45.8</x:v>
       </x:c>
       <x:c r="F58" s="17" t="n">
-        <x:v>593.8</x:v>
+        <x:v>566.3</x:v>
       </x:c>
       <x:c r="G58" s="17" t="n">
-        <x:v>3.4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H58" s="17" t="n">
-        <x:v>2.5</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="I58" s="17" t="n">
-        <x:v>12.1</x:v>
+        <x:v>16.9</x:v>
       </x:c>
       <x:c r="J58" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="K58" s="17" t="n">
         <x:v>1.4</x:v>
       </x:c>
       <x:c r="L58" s="17" t="n">
-        <x:v>122.6</x:v>
+        <x:v>119.9</x:v>
       </x:c>
       <x:c r="M58" s="17" t="n">
-        <x:v>100.4</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="N58" s="26" t="n">
-        <x:v>78.1</x:v>
+        <x:v>74.1</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
@@ -12415,43 +12482,43 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" s="20" t="str">
-        <x:v>KC Concepcion</x:v>
+        <x:v>Calvin Ridley</x:v>
       </x:c>
       <x:c r="C59" s="16" t="str">
-        <x:v>CLE</x:v>
+        <x:v>TEN</x:v>
       </x:c>
       <x:c r="D59" s="17" t="n">
-        <x:v>74.4</x:v>
+        <x:v>71.3</x:v>
       </x:c>
       <x:c r="E59" s="17" t="n">
-        <x:v>45.8</x:v>
+        <x:v>37.3</x:v>
       </x:c>
       <x:c r="F59" s="17" t="n">
-        <x:v>566.3</x:v>
+        <x:v>589.7</x:v>
       </x:c>
       <x:c r="G59" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H59" s="17" t="n">
-        <x:v>3.2</x:v>
+        <x:v>3.6</x:v>
       </x:c>
       <x:c r="I59" s="17" t="n">
-        <x:v>16.9</x:v>
+        <x:v>23.6</x:v>
       </x:c>
       <x:c r="J59" s="17" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="K59" s="17" t="n">
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="K59" s="17" t="n">
-        <x:v>1.4</x:v>
-      </x:c>
       <x:c r="L59" s="17" t="n">
-        <x:v>119.9</x:v>
+        <x:v>117.5</x:v>
       </x:c>
       <x:c r="M59" s="17" t="n">
-        <x:v>97</x:v>
+        <x:v>98.8</x:v>
       </x:c>
       <x:c r="N59" s="26" t="n">
-        <x:v>74.1</x:v>
+        <x:v>80.2</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
@@ -12459,43 +12526,43 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" s="20" t="str">
-        <x:v>Calvin Ridley</x:v>
+        <x:v>Jalen Nailor</x:v>
       </x:c>
       <x:c r="C60" s="16" t="str">
-        <x:v>TEN</x:v>
+        <x:v>LV</x:v>
       </x:c>
       <x:c r="D60" s="17" t="n">
-        <x:v>71.3</x:v>
+        <x:v>66.5</x:v>
       </x:c>
       <x:c r="E60" s="17" t="n">
-        <x:v>37.3</x:v>
+        <x:v>39.9</x:v>
       </x:c>
       <x:c r="F60" s="17" t="n">
-        <x:v>589.7</x:v>
+        <x:v>532.1</x:v>
       </x:c>
       <x:c r="G60" s="17" t="n">
-        <x:v>2.5</x:v>
+        <x:v>3.6</x:v>
       </x:c>
       <x:c r="H60" s="17" t="n">
-        <x:v>3.6</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I60" s="17" t="n">
-        <x:v>23.6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J60" s="17" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K60" s="17" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="L60" s="17" t="n">
-        <x:v>117.5</x:v>
+        <x:v>115.1</x:v>
       </x:c>
       <x:c r="M60" s="17" t="n">
-        <x:v>98.8</x:v>
+        <x:v>95.2</x:v>
       </x:c>
       <x:c r="N60" s="26" t="n">
-        <x:v>80.2</x:v>
+        <x:v>75.2</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
@@ -12503,43 +12570,43 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" s="20" t="str">
-        <x:v>Jalen Nailor</x:v>
+        <x:v>Makai Lemon</x:v>
       </x:c>
       <x:c r="C61" s="16" t="str">
-        <x:v>LV</x:v>
+        <x:v>PHI</x:v>
       </x:c>
       <x:c r="D61" s="17" t="n">
-        <x:v>66.5</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E61" s="17" t="n">
-        <x:v>39.9</x:v>
+        <x:v>39.6</x:v>
       </x:c>
       <x:c r="F61" s="17" t="n">
-        <x:v>532.1</x:v>
+        <x:v>529.6</x:v>
       </x:c>
       <x:c r="G61" s="17" t="n">
-        <x:v>3.6</x:v>
+        <x:v>3.03</x:v>
       </x:c>
       <x:c r="H61" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="I61" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>12.1</x:v>
       </x:c>
       <x:c r="J61" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K61" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="L61" s="17" t="n">
-        <x:v>115.1</x:v>
+        <x:v>109.2</x:v>
       </x:c>
       <x:c r="M61" s="17" t="n">
-        <x:v>95.2</x:v>
+        <x:v>89.3</x:v>
       </x:c>
       <x:c r="N61" s="26" t="n">
-        <x:v>75.2</x:v>
+        <x:v>69.5</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
@@ -13515,43 +13582,43 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="B84" s="20" t="str">
-        <x:v>Jack Bech</x:v>
+        <x:v>Dontayvion Wicks</x:v>
       </x:c>
       <x:c r="C84" s="16" t="str">
-        <x:v>LV</x:v>
+        <x:v>PHI</x:v>
       </x:c>
       <x:c r="D84" s="17" t="n">
-        <x:v>49.8</x:v>
+        <x:v>50.1</x:v>
       </x:c>
       <x:c r="E84" s="17" t="n">
-        <x:v>31.6</x:v>
+        <x:v>30.6</x:v>
       </x:c>
       <x:c r="F84" s="17" t="n">
-        <x:v>372.5</x:v>
+        <x:v>330.3</x:v>
       </x:c>
       <x:c r="G84" s="17" t="n">
-        <x:v>1.4</x:v>
+        <x:v>2.18</x:v>
       </x:c>
       <x:c r="H84" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I84" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="J84" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K84" s="17" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L84" s="17" t="n">
-        <x:v>76.8</x:v>
+        <x:v>77.1</x:v>
       </x:c>
       <x:c r="M84" s="17" t="n">
-        <x:v>61</x:v>
+        <x:v>61.8</x:v>
       </x:c>
       <x:c r="N84" s="26" t="n">
-        <x:v>45.2</x:v>
+        <x:v>46.5</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
@@ -13559,43 +13626,43 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="B85" s="20" t="str">
-        <x:v>Cooper Kupp</x:v>
+        <x:v>Jack Bech</x:v>
       </x:c>
       <x:c r="C85" s="16" t="str">
-        <x:v>SEA</x:v>
+        <x:v>LV</x:v>
       </x:c>
       <x:c r="D85" s="17" t="n">
-        <x:v>45</x:v>
+        <x:v>49.8</x:v>
       </x:c>
       <x:c r="E85" s="17" t="n">
-        <x:v>29.1</x:v>
+        <x:v>31.6</x:v>
       </x:c>
       <x:c r="F85" s="17" t="n">
-        <x:v>357.3</x:v>
+        <x:v>372.5</x:v>
       </x:c>
       <x:c r="G85" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="H85" s="17" t="n">
-        <x:v>0.7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I85" s="17" t="n">
-        <x:v>2.4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J85" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K85" s="17" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="L85" s="17" t="n">
-        <x:v>76.5</x:v>
+        <x:v>76.8</x:v>
       </x:c>
       <x:c r="M85" s="17" t="n">
-        <x:v>61.9</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="N85" s="26" t="n">
-        <x:v>47.4</x:v>
+        <x:v>45.2</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
@@ -13603,43 +13670,43 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="B86" s="20" t="str">
-        <x:v>Ashton Dulin</x:v>
+        <x:v>Cooper Kupp</x:v>
       </x:c>
       <x:c r="C86" s="16" t="str">
-        <x:v>IND</x:v>
+        <x:v>SEA</x:v>
       </x:c>
       <x:c r="D86" s="17" t="n">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E86" s="17" t="n">
-        <x:v>23.2</x:v>
+        <x:v>29.1</x:v>
       </x:c>
       <x:c r="F86" s="17" t="n">
-        <x:v>373.3</x:v>
+        <x:v>357.3</x:v>
       </x:c>
       <x:c r="G86" s="17" t="n">
-        <x:v>1.7</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="H86" s="17" t="n">
-        <x:v>5.2</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="I86" s="17" t="n">
-        <x:v>49.2</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="J86" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K86" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="L86" s="17" t="n">
-        <x:v>76.1</x:v>
+        <x:v>76.5</x:v>
       </x:c>
       <x:c r="M86" s="17" t="n">
-        <x:v>64.4</x:v>
+        <x:v>61.9</x:v>
       </x:c>
       <x:c r="N86" s="26" t="n">
-        <x:v>52.8</x:v>
+        <x:v>47.4</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
@@ -13647,43 +13714,43 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="B87" s="20" t="str">
-        <x:v>Kayshon Boutte</x:v>
+        <x:v>Ashton Dulin</x:v>
       </x:c>
       <x:c r="C87" s="16" t="str">
-        <x:v>NE</x:v>
+        <x:v>IND</x:v>
       </x:c>
       <x:c r="D87" s="17" t="n">
-        <x:v>33.7</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E87" s="17" t="n">
-        <x:v>22.2</x:v>
+        <x:v>23.2</x:v>
       </x:c>
       <x:c r="F87" s="17" t="n">
-        <x:v>337.5</x:v>
+        <x:v>373.3</x:v>
       </x:c>
       <x:c r="G87" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>1.7</x:v>
       </x:c>
       <x:c r="H87" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="I87" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>49.2</x:v>
       </x:c>
       <x:c r="J87" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="K87" s="17" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="L87" s="17" t="n">
-        <x:v>73.9</x:v>
+        <x:v>76.1</x:v>
       </x:c>
       <x:c r="M87" s="17" t="n">
-        <x:v>62.8</x:v>
+        <x:v>64.4</x:v>
       </x:c>
       <x:c r="N87" s="26" t="n">
-        <x:v>51.8</x:v>
+        <x:v>52.8</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
@@ -13691,22 +13758,22 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="B88" s="20" t="str">
-        <x:v>Tyquan Thornton</x:v>
+        <x:v>Kayshon Boutte</x:v>
       </x:c>
       <x:c r="C88" s="16" t="str">
-        <x:v>KC</x:v>
+        <x:v>NE</x:v>
       </x:c>
       <x:c r="D88" s="17" t="n">
-        <x:v>40.2</x:v>
+        <x:v>33.7</x:v>
       </x:c>
       <x:c r="E88" s="17" t="n">
-        <x:v>20.3</x:v>
+        <x:v>22.2</x:v>
       </x:c>
       <x:c r="F88" s="17" t="n">
-        <x:v>376.1</x:v>
+        <x:v>337.5</x:v>
       </x:c>
       <x:c r="G88" s="17" t="n">
-        <x:v>2.6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H88" s="17" t="n">
         <x:v>0</x:v>
@@ -13721,13 +13788,13 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="L88" s="17" t="n">
-        <x:v>73.6</x:v>
+        <x:v>73.9</x:v>
       </x:c>
       <x:c r="M88" s="17" t="n">
-        <x:v>63.5</x:v>
+        <x:v>62.8</x:v>
       </x:c>
       <x:c r="N88" s="26" t="n">
-        <x:v>53.3</x:v>
+        <x:v>51.8</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
@@ -13735,22 +13802,22 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="B89" s="20" t="str">
-        <x:v>Devontez Walker</x:v>
+        <x:v>Tyquan Thornton</x:v>
       </x:c>
       <x:c r="C89" s="16" t="str">
-        <x:v>BAL</x:v>
+        <x:v>KC</x:v>
       </x:c>
       <x:c r="D89" s="17" t="n">
-        <x:v>40.3</x:v>
+        <x:v>40.2</x:v>
       </x:c>
       <x:c r="E89" s="17" t="n">
-        <x:v>25.3</x:v>
+        <x:v>20.3</x:v>
       </x:c>
       <x:c r="F89" s="17" t="n">
-        <x:v>337.3</x:v>
+        <x:v>376.1</x:v>
       </x:c>
       <x:c r="G89" s="17" t="n">
-        <x:v>2.2</x:v>
+        <x:v>2.6</x:v>
       </x:c>
       <x:c r="H89" s="17" t="n">
         <x:v>0</x:v>
@@ -13762,16 +13829,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K89" s="17" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L89" s="17" t="n">
-        <x:v>71.5</x:v>
+        <x:v>73.6</x:v>
       </x:c>
       <x:c r="M89" s="17" t="n">
-        <x:v>58.9</x:v>
+        <x:v>63.5</x:v>
       </x:c>
       <x:c r="N89" s="26" t="n">
-        <x:v>46.2</x:v>
+        <x:v>53.3</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
@@ -13779,43 +13846,43 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B90" s="20" t="str">
-        <x:v>Ryan Flournoy</x:v>
+        <x:v>Devontez Walker</x:v>
       </x:c>
       <x:c r="C90" s="16" t="str">
-        <x:v>DAL</x:v>
+        <x:v>BAL</x:v>
       </x:c>
       <x:c r="D90" s="17" t="n">
-        <x:v>39.3</x:v>
+        <x:v>40.3</x:v>
       </x:c>
       <x:c r="E90" s="17" t="n">
-        <x:v>26.1</x:v>
+        <x:v>25.3</x:v>
       </x:c>
       <x:c r="F90" s="17" t="n">
-        <x:v>304.7</x:v>
+        <x:v>337.3</x:v>
       </x:c>
       <x:c r="G90" s="17" t="n">
         <x:v>2.2</x:v>
       </x:c>
       <x:c r="H90" s="17" t="n">
-        <x:v>2.5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I90" s="17" t="n">
-        <x:v>13.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J90" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K90" s="17" t="n">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="L90" s="17" t="n">
-        <x:v>71.2</x:v>
+        <x:v>71.5</x:v>
       </x:c>
       <x:c r="M90" s="17" t="n">
-        <x:v>58.1</x:v>
+        <x:v>58.9</x:v>
       </x:c>
       <x:c r="N90" s="26" t="n">
-        <x:v>45.1</x:v>
+        <x:v>46.2</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15" hidden="0" customHeight="1">
@@ -13823,43 +13890,43 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="B91" s="20" t="str">
-        <x:v>Caleb Douglas</x:v>
+        <x:v>Ryan Flournoy</x:v>
       </x:c>
       <x:c r="C91" s="16" t="str">
-        <x:v>MIA</x:v>
+        <x:v>DAL</x:v>
       </x:c>
       <x:c r="D91" s="17" t="n">
-        <x:v>45.6</x:v>
+        <x:v>39.3</x:v>
       </x:c>
       <x:c r="E91" s="17" t="n">
-        <x:v>27.6</x:v>
+        <x:v>26.1</x:v>
       </x:c>
       <x:c r="F91" s="17" t="n">
-        <x:v>332.3</x:v>
+        <x:v>304.7</x:v>
       </x:c>
       <x:c r="G91" s="17" t="n">
-        <x:v>1.8</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H91" s="17" t="n">
-        <x:v>1.4</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="I91" s="17" t="n">
-        <x:v>7.8</x:v>
+        <x:v>13.9</x:v>
       </x:c>
       <x:c r="J91" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="K91" s="17" t="n">
-        <x:v>0.6</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="L91" s="17" t="n">
         <x:v>71.2</x:v>
       </x:c>
       <x:c r="M91" s="17" t="n">
-        <x:v>57.4</x:v>
+        <x:v>58.1</x:v>
       </x:c>
       <x:c r="N91" s="26" t="n">
-        <x:v>43.6</x:v>
+        <x:v>45.1</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
@@ -13867,43 +13934,43 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="B92" s="20" t="str">
-        <x:v>Elic Ayomanor</x:v>
+        <x:v>Caleb Douglas</x:v>
       </x:c>
       <x:c r="C92" s="16" t="str">
-        <x:v>TEN</x:v>
+        <x:v>MIA</x:v>
       </x:c>
       <x:c r="D92" s="17" t="n">
-        <x:v>47.9</x:v>
+        <x:v>45.6</x:v>
       </x:c>
       <x:c r="E92" s="17" t="n">
-        <x:v>24.4</x:v>
+        <x:v>27.6</x:v>
       </x:c>
       <x:c r="F92" s="17" t="n">
-        <x:v>315.9</x:v>
+        <x:v>332.3</x:v>
       </x:c>
       <x:c r="G92" s="17" t="n">
-        <x:v>2.5</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="H92" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="I92" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>7.8</x:v>
       </x:c>
       <x:c r="J92" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K92" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.6</x:v>
       </x:c>
       <x:c r="L92" s="17" t="n">
-        <x:v>71</x:v>
+        <x:v>71.2</x:v>
       </x:c>
       <x:c r="M92" s="17" t="n">
-        <x:v>58.8</x:v>
+        <x:v>57.4</x:v>
       </x:c>
       <x:c r="N92" s="26" t="n">
-        <x:v>46.6</x:v>
+        <x:v>43.6</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15" hidden="0" customHeight="1">
@@ -13911,43 +13978,43 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="B93" s="20" t="str">
-        <x:v>Dontayvion Wicks</x:v>
+        <x:v>Elic Ayomanor</x:v>
       </x:c>
       <x:c r="C93" s="16" t="str">
-        <x:v>PHI</x:v>
+        <x:v>TEN</x:v>
       </x:c>
       <x:c r="D93" s="17" t="n">
-        <x:v>46.1</x:v>
+        <x:v>47.9</x:v>
       </x:c>
       <x:c r="E93" s="17" t="n">
-        <x:v>28.2</x:v>
+        <x:v>24.4</x:v>
       </x:c>
       <x:c r="F93" s="17" t="n">
-        <x:v>298.2</x:v>
+        <x:v>315.9</x:v>
       </x:c>
       <x:c r="G93" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="H93" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I93" s="17" t="n">
-        <x:v>6.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J93" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K93" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L93" s="17" t="n">
-        <x:v>70.6</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="M93" s="17" t="n">
-        <x:v>56.6</x:v>
+        <x:v>58.8</x:v>
       </x:c>
       <x:c r="N93" s="26" t="n">
-        <x:v>42.5</x:v>
+        <x:v>46.6</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="15" hidden="0" customHeight="1">
@@ -13999,22 +14066,22 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="B95" s="20" t="str">
-        <x:v>Mack Hollins</x:v>
+        <x:v>Hollywood Brown</x:v>
       </x:c>
       <x:c r="C95" s="16" t="str">
-        <x:v>NE</x:v>
+        <x:v>PHI</x:v>
       </x:c>
       <x:c r="D95" s="17" t="n">
-        <x:v>35</x:v>
+        <x:v>40.5</x:v>
       </x:c>
       <x:c r="E95" s="17" t="n">
-        <x:v>24.8</x:v>
+        <x:v>25.2</x:v>
       </x:c>
       <x:c r="F95" s="17" t="n">
-        <x:v>295.3</x:v>
+        <x:v>295.8</x:v>
       </x:c>
       <x:c r="G95" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H95" s="17" t="n">
         <x:v>0</x:v>
@@ -14026,16 +14093,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K95" s="17" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L95" s="17" t="n">
-        <x:v>66.4</x:v>
+        <x:v>67.8</x:v>
       </x:c>
       <x:c r="M95" s="17" t="n">
-        <x:v>54</x:v>
+        <x:v>55.2</x:v>
       </x:c>
       <x:c r="N95" s="26" t="n">
-        <x:v>41.6</x:v>
+        <x:v>42.6</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="15" hidden="0" customHeight="1">
@@ -14043,43 +14110,43 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="B96" s="20" t="str">
-        <x:v>Travis Hunter</x:v>
+        <x:v>Mack Hollins</x:v>
       </x:c>
       <x:c r="C96" s="16" t="str">
-        <x:v>JAX</x:v>
+        <x:v>NE</x:v>
       </x:c>
       <x:c r="D96" s="17" t="n">
-        <x:v>38.5</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E96" s="17" t="n">
-        <x:v>22.9</x:v>
+        <x:v>24.8</x:v>
       </x:c>
       <x:c r="F96" s="17" t="n">
-        <x:v>286.4</x:v>
+        <x:v>295.3</x:v>
       </x:c>
       <x:c r="G96" s="17" t="n">
-        <x:v>2.2</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="H96" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I96" s="17" t="n">
-        <x:v>10.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J96" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K96" s="17" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="L96" s="17" t="n">
-        <x:v>65.5</x:v>
+        <x:v>66.4</x:v>
       </x:c>
       <x:c r="M96" s="17" t="n">
         <x:v>54</x:v>
       </x:c>
       <x:c r="N96" s="26" t="n">
-        <x:v>42.6</x:v>
+        <x:v>41.6</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="15" hidden="0" customHeight="1">
@@ -14087,43 +14154,43 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="B97" s="20" t="str">
-        <x:v>Joshua Palmer</x:v>
+        <x:v>Travis Hunter</x:v>
       </x:c>
       <x:c r="C97" s="16" t="str">
-        <x:v>BUF</x:v>
+        <x:v>JAX</x:v>
       </x:c>
       <x:c r="D97" s="17" t="n">
-        <x:v>37.6</x:v>
+        <x:v>38.5</x:v>
       </x:c>
       <x:c r="E97" s="17" t="n">
-        <x:v>24.7</x:v>
+        <x:v>22.9</x:v>
       </x:c>
       <x:c r="F97" s="17" t="n">
-        <x:v>301</x:v>
+        <x:v>286.4</x:v>
       </x:c>
       <x:c r="G97" s="17" t="n">
-        <x:v>1.8</x:v>
+        <x:v>2.2</x:v>
       </x:c>
       <x:c r="H97" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I97" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>10.9</x:v>
       </x:c>
       <x:c r="J97" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="K97" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="L97" s="17" t="n">
-        <x:v>65.3</x:v>
+        <x:v>65.5</x:v>
       </x:c>
       <x:c r="M97" s="17" t="n">
-        <x:v>52.9</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="N97" s="26" t="n">
-        <x:v>40.5</x:v>
+        <x:v>42.6</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15" hidden="0" customHeight="1">
@@ -14131,22 +14198,22 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="B98" s="20" t="str">
-        <x:v>Jalen Tolbert</x:v>
+        <x:v>Joshua Palmer</x:v>
       </x:c>
       <x:c r="C98" s="16" t="str">
-        <x:v>MIA</x:v>
+        <x:v>BUF</x:v>
       </x:c>
       <x:c r="D98" s="17" t="n">
-        <x:v>40.4</x:v>
+        <x:v>37.6</x:v>
       </x:c>
       <x:c r="E98" s="17" t="n">
-        <x:v>26</x:v>
+        <x:v>24.7</x:v>
       </x:c>
       <x:c r="F98" s="17" t="n">
-        <x:v>309.1</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="G98" s="17" t="n">
-        <x:v>1.45</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="H98" s="17" t="n">
         <x:v>0</x:v>
@@ -14158,16 +14225,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K98" s="17" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="L98" s="17" t="n">
-        <x:v>64.8</x:v>
+        <x:v>65.3</x:v>
       </x:c>
       <x:c r="M98" s="17" t="n">
-        <x:v>51.8</x:v>
+        <x:v>52.9</x:v>
       </x:c>
       <x:c r="N98" s="26" t="n">
-        <x:v>38.8</x:v>
+        <x:v>40.5</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="15" hidden="0" customHeight="1">
@@ -14175,22 +14242,22 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B99" s="20" t="str">
-        <x:v>Hollywood Brown</x:v>
+        <x:v>Jalen Tolbert</x:v>
       </x:c>
       <x:c r="C99" s="16" t="str">
-        <x:v>PHI</x:v>
+        <x:v>MIA</x:v>
       </x:c>
       <x:c r="D99" s="17" t="n">
-        <x:v>38.5</x:v>
+        <x:v>40.4</x:v>
       </x:c>
       <x:c r="E99" s="17" t="n">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F99" s="17" t="n">
-        <x:v>279.7</x:v>
+        <x:v>309.1</x:v>
       </x:c>
       <x:c r="G99" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>1.45</x:v>
       </x:c>
       <x:c r="H99" s="17" t="n">
         <x:v>0</x:v>
@@ -14202,16 +14269,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K99" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="L99" s="17" t="n">
-        <x:v>64.5</x:v>
+        <x:v>64.8</x:v>
       </x:c>
       <x:c r="M99" s="17" t="n">
-        <x:v>52.6</x:v>
+        <x:v>51.8</x:v>
       </x:c>
       <x:c r="N99" s="26" t="n">
-        <x:v>40.6</x:v>
+        <x:v>38.8</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15" hidden="0" customHeight="1">
@@ -17519,43 +17586,43 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="B175" s="20" t="str">
-        <x:v>Derius Davis</x:v>
+        <x:v>Darius Cooper</x:v>
       </x:c>
       <x:c r="C175" s="16" t="str">
-        <x:v>LAC</x:v>
+        <x:v>PHI</x:v>
       </x:c>
       <x:c r="D175" s="17" t="n">
-        <x:v>3.5</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="E175" s="17" t="n">
-        <x:v>2.4</x:v>
+        <x:v>3.1</x:v>
       </x:c>
       <x:c r="F175" s="17" t="n">
-        <x:v>25.3</x:v>
+        <x:v>36.1</x:v>
       </x:c>
       <x:c r="G175" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.19</x:v>
       </x:c>
       <x:c r="H175" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I175" s="17" t="n">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J175" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K175" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L175" s="17" t="n">
-        <x:v>7.3</x:v>
+        <x:v>7.8</x:v>
       </x:c>
       <x:c r="M175" s="17" t="n">
-        <x:v>6.1</x:v>
+        <x:v>6.3</x:v>
       </x:c>
       <x:c r="N175" s="26" t="n">
-        <x:v>4.9</x:v>
+        <x:v>4.8</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="15" hidden="0" customHeight="1">
@@ -17563,43 +17630,43 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="B176" s="20" t="str">
-        <x:v>Tyrell Shavers</x:v>
+        <x:v>Derius Davis</x:v>
       </x:c>
       <x:c r="C176" s="16" t="str">
-        <x:v>BUF</x:v>
+        <x:v>LAC</x:v>
       </x:c>
       <x:c r="D176" s="17" t="n">
-        <x:v>4.1</x:v>
+        <x:v>3.5</x:v>
       </x:c>
       <x:c r="E176" s="17" t="n">
-        <x:v>2.7</x:v>
+        <x:v>2.4</x:v>
       </x:c>
       <x:c r="F176" s="17" t="n">
-        <x:v>33.2</x:v>
+        <x:v>25.3</x:v>
       </x:c>
       <x:c r="G176" s="17" t="n">
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="H176" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="I176" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="J176" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="K176" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L176" s="17" t="n">
         <x:v>7.3</x:v>
       </x:c>
       <x:c r="M176" s="17" t="n">
-        <x:v>5.9</x:v>
+        <x:v>6.1</x:v>
       </x:c>
       <x:c r="N176" s="26" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4.9</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="15" hidden="0" customHeight="1">
@@ -17607,19 +17674,19 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="B177" s="20" t="str">
-        <x:v>Cody White</x:v>
+        <x:v>Tyrell Shavers</x:v>
       </x:c>
       <x:c r="C177" s="16" t="str">
-        <x:v>SEA</x:v>
+        <x:v>BUF</x:v>
       </x:c>
       <x:c r="D177" s="17" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4.1</x:v>
       </x:c>
       <x:c r="E177" s="17" t="n">
-        <x:v>2.8</x:v>
+        <x:v>2.7</x:v>
       </x:c>
       <x:c r="F177" s="17" t="n">
-        <x:v>32.6</x:v>
+        <x:v>33.2</x:v>
       </x:c>
       <x:c r="G177" s="17" t="n">
         <x:v>0.2</x:v>
@@ -17637,13 +17704,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L177" s="17" t="n">
-        <x:v>7.2</x:v>
+        <x:v>7.3</x:v>
       </x:c>
       <x:c r="M177" s="17" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5.9</x:v>
       </x:c>
       <x:c r="N177" s="26" t="n">
-        <x:v>4.3</x:v>
+        <x:v>4.5</x:v>
       </x:c>
     </x:row>
     <x:row r="178" ht="15" hidden="0" customHeight="1">
@@ -17651,43 +17718,43 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B178" s="20" t="str">
-        <x:v>Malachi Corley</x:v>
+        <x:v>Cody White</x:v>
       </x:c>
       <x:c r="C178" s="16" t="str">
-        <x:v>CLE</x:v>
+        <x:v>SEA</x:v>
       </x:c>
       <x:c r="D178" s="17" t="n">
-        <x:v>1.2</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="E178" s="17" t="n">
-        <x:v>0.8</x:v>
+        <x:v>2.8</x:v>
       </x:c>
       <x:c r="F178" s="17" t="n">
-        <x:v>7.6</x:v>
+        <x:v>32.6</x:v>
       </x:c>
       <x:c r="G178" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H178" s="17" t="n">
-        <x:v>6.4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I178" s="17" t="n">
-        <x:v>42.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J178" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K178" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L178" s="17" t="n">
-        <x:v>7</x:v>
+        <x:v>7.2</x:v>
       </x:c>
       <x:c r="M178" s="17" t="n">
-        <x:v>6.6</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="N178" s="26" t="n">
-        <x:v>6.3</x:v>
+        <x:v>4.3</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="15" hidden="0" customHeight="1">
@@ -17695,43 +17762,43 @@
         <x:v>178</x:v>
       </x:c>
       <x:c r="B179" s="20" t="str">
-        <x:v>Laquon Treadwell</x:v>
+        <x:v>Malachi Corley</x:v>
       </x:c>
       <x:c r="C179" s="16" t="str">
-        <x:v>IND</x:v>
+        <x:v>CLE</x:v>
       </x:c>
       <x:c r="D179" s="17" t="n">
-        <x:v>4.3</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="E179" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="F179" s="17" t="n">
-        <x:v>28.8</x:v>
+        <x:v>7.6</x:v>
       </x:c>
       <x:c r="G179" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H179" s="17" t="n">
+        <x:v>6.4</x:v>
+      </x:c>
+      <x:c r="I179" s="17" t="n">
+        <x:v>42.1</x:v>
+      </x:c>
+      <x:c r="J179" s="17" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="H179" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I179" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J179" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="K179" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L179" s="17" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="M179" s="17" t="n">
-        <x:v>5.5</x:v>
+        <x:v>6.6</x:v>
       </x:c>
       <x:c r="N179" s="26" t="n">
-        <x:v>4</x:v>
+        <x:v>6.3</x:v>
       </x:c>
     </x:row>
     <x:row r="180" ht="15" hidden="0" customHeight="1">
@@ -17739,22 +17806,22 @@
         <x:v>179</x:v>
       </x:c>
       <x:c r="B180" s="20" t="str">
-        <x:v>Isaiah Hodgins</x:v>
+        <x:v>Laquon Treadwell</x:v>
       </x:c>
       <x:c r="C180" s="16" t="str">
-        <x:v>NYG</x:v>
+        <x:v>IND</x:v>
       </x:c>
       <x:c r="D180" s="17" t="n">
-        <x:v>4.6</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="E180" s="17" t="n">
-        <x:v>2.6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F180" s="17" t="n">
-        <x:v>32.5</x:v>
+        <x:v>28.8</x:v>
       </x:c>
       <x:c r="G180" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H180" s="17" t="n">
         <x:v>0</x:v>
@@ -17769,13 +17836,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L180" s="17" t="n">
-        <x:v>6.7</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="M180" s="17" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="N180" s="26" t="n">
-        <x:v>4.1</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="181" ht="15" hidden="0" customHeight="1">
@@ -17783,43 +17850,43 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="B181" s="20" t="str">
-        <x:v>Mason Tipton</x:v>
+        <x:v>Isaiah Hodgins</x:v>
       </x:c>
       <x:c r="C181" s="16" t="str">
-        <x:v>NO</x:v>
+        <x:v>NYG</x:v>
       </x:c>
       <x:c r="D181" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="E181" s="17" t="n">
-        <x:v>1.3</x:v>
+        <x:v>2.6</x:v>
       </x:c>
       <x:c r="F181" s="17" t="n">
-        <x:v>13.8</x:v>
+        <x:v>32.5</x:v>
       </x:c>
       <x:c r="G181" s="17" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="H181" s="17" t="n">
-        <x:v>4.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I181" s="17" t="n">
-        <x:v>23.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J181" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K181" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L181" s="17" t="n">
-        <x:v>6.4</x:v>
+        <x:v>6.7</x:v>
       </x:c>
       <x:c r="M181" s="17" t="n">
-        <x:v>5.8</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="N181" s="26" t="n">
-        <x:v>5.1</x:v>
+        <x:v>4.1</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="15" hidden="0" customHeight="1">
@@ -17827,43 +17894,43 @@
         <x:v>181</x:v>
       </x:c>
       <x:c r="B182" s="20" t="str">
-        <x:v>Jonathan Mingo</x:v>
+        <x:v>Mason Tipton</x:v>
       </x:c>
       <x:c r="C182" s="16" t="str">
-        <x:v>DAL</x:v>
+        <x:v>NO</x:v>
       </x:c>
       <x:c r="D182" s="17" t="n">
-        <x:v>3.3</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="E182" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>1.3</x:v>
       </x:c>
       <x:c r="F182" s="17" t="n">
-        <x:v>27.9</x:v>
+        <x:v>13.8</x:v>
       </x:c>
       <x:c r="G182" s="17" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="H182" s="17" t="n">
+        <x:v>4.3</x:v>
+      </x:c>
+      <x:c r="I182" s="17" t="n">
+        <x:v>23.3</x:v>
+      </x:c>
+      <x:c r="J182" s="17" t="n">
         <x:v>0.2</x:v>
       </x:c>
-      <x:c r="H182" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I182" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J182" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="K182" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L182" s="17" t="n">
-        <x:v>6</x:v>
+        <x:v>6.4</x:v>
       </x:c>
       <x:c r="M182" s="17" t="n">
-        <x:v>5</x:v>
+        <x:v>5.8</x:v>
       </x:c>
       <x:c r="N182" s="26" t="n">
-        <x:v>4</x:v>
+        <x:v>5.1</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="15" hidden="0" customHeight="1">
@@ -17871,43 +17938,43 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B183" s="20" t="str">
-        <x:v>David Moore</x:v>
+        <x:v>Jonathan Mingo</x:v>
       </x:c>
       <x:c r="C183" s="16" t="str">
-        <x:v>CAR</x:v>
+        <x:v>DAL</x:v>
       </x:c>
       <x:c r="D183" s="17" t="n">
-        <x:v>3.1</x:v>
+        <x:v>3.3</x:v>
       </x:c>
       <x:c r="E183" s="17" t="n">
-        <x:v>1.8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F183" s="17" t="n">
-        <x:v>19.5</x:v>
+        <x:v>27.9</x:v>
       </x:c>
       <x:c r="G183" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H183" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I183" s="17" t="n">
-        <x:v>11.4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J183" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K183" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L183" s="17" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="M183" s="17" t="n">
-        <x:v>5.1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N183" s="26" t="n">
-        <x:v>4.2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="15" hidden="0" customHeight="1">
@@ -17915,19 +17982,19 @@
         <x:v>183</x:v>
       </x:c>
       <x:c r="B184" s="20" t="str">
-        <x:v>Kaden Wetjen</x:v>
+        <x:v>David Moore</x:v>
       </x:c>
       <x:c r="C184" s="16" t="str">
-        <x:v>PIT</x:v>
+        <x:v>CAR</x:v>
       </x:c>
       <x:c r="D184" s="17" t="n">
-        <x:v>2.9</x:v>
+        <x:v>3.1</x:v>
       </x:c>
       <x:c r="E184" s="17" t="n">
-        <x:v>1.7</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="F184" s="17" t="n">
-        <x:v>17.5</x:v>
+        <x:v>19.5</x:v>
       </x:c>
       <x:c r="G184" s="17" t="n">
         <x:v>0.1</x:v>
@@ -17942,16 +18009,16 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="K184" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="L184" s="17" t="n">
-        <x:v>5.7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M184" s="17" t="n">
-        <x:v>4.8</x:v>
+        <x:v>5.1</x:v>
       </x:c>
       <x:c r="N184" s="26" t="n">
-        <x:v>4</x:v>
+        <x:v>4.2</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="15" hidden="0" customHeight="1">
@@ -17959,31 +18026,31 @@
         <x:v>184</x:v>
       </x:c>
       <x:c r="B185" s="20" t="str">
-        <x:v>Chase Roberts</x:v>
+        <x:v>Kaden Wetjen</x:v>
       </x:c>
       <x:c r="C185" s="16" t="str">
-        <x:v>LV</x:v>
+        <x:v>PIT</x:v>
       </x:c>
       <x:c r="D185" s="17" t="n">
-        <x:v>3.8</x:v>
+        <x:v>2.9</x:v>
       </x:c>
       <x:c r="E185" s="17" t="n">
-        <x:v>2.3</x:v>
+        <x:v>1.7</x:v>
       </x:c>
       <x:c r="F185" s="17" t="n">
-        <x:v>28.5</x:v>
+        <x:v>17.5</x:v>
       </x:c>
       <x:c r="G185" s="17" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="H185" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="I185" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>11.4</x:v>
       </x:c>
       <x:c r="J185" s="17" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="K185" s="17" t="n">
         <x:v>0</x:v>
@@ -17992,10 +18059,10 @@
         <x:v>5.7</x:v>
       </x:c>
       <x:c r="M185" s="17" t="n">
-        <x:v>4.5</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="N185" s="26" t="n">
-        <x:v>3.3</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="186" ht="15" hidden="0" customHeight="1">
@@ -18003,22 +18070,22 @@
         <x:v>185</x:v>
       </x:c>
       <x:c r="B186" s="20" t="str">
-        <x:v>Tyler Johnson</x:v>
+        <x:v>Chase Roberts</x:v>
       </x:c>
       <x:c r="C186" s="16" t="str">
-        <x:v>DAL</x:v>
+        <x:v>LV</x:v>
       </x:c>
       <x:c r="D186" s="17" t="n">
-        <x:v>3.1</x:v>
+        <x:v>3.8</x:v>
       </x:c>
       <x:c r="E186" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>2.3</x:v>
       </x:c>
       <x:c r="F186" s="17" t="n">
-        <x:v>24.3</x:v>
+        <x:v>28.5</x:v>
       </x:c>
       <x:c r="G186" s="17" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="H186" s="17" t="n">
         <x:v>0</x:v>
@@ -18033,10 +18100,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L186" s="17" t="n">
-        <x:v>5.4</x:v>
+        <x:v>5.7</x:v>
       </x:c>
       <x:c r="M186" s="17" t="n">
-        <x:v>4.4</x:v>
+        <x:v>4.5</x:v>
       </x:c>
       <x:c r="N186" s="26" t="n">
         <x:v>3.3</x:v>
@@ -18047,22 +18114,22 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="B187" s="20" t="str">
-        <x:v>Dane Key</x:v>
+        <x:v>Tyler Johnson</x:v>
       </x:c>
       <x:c r="C187" s="16" t="str">
-        <x:v>DEN</x:v>
+        <x:v>DAL</x:v>
       </x:c>
       <x:c r="D187" s="17" t="n">
-        <x:v>3.3</x:v>
+        <x:v>3.1</x:v>
       </x:c>
       <x:c r="E187" s="17" t="n">
-        <x:v>2.1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F187" s="17" t="n">
-        <x:v>25.3</x:v>
+        <x:v>24.3</x:v>
       </x:c>
       <x:c r="G187" s="17" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H187" s="17" t="n">
         <x:v>0</x:v>
@@ -18080,7 +18147,7 @@
         <x:v>5.4</x:v>
       </x:c>
       <x:c r="M187" s="17" t="n">
-        <x:v>4.3</x:v>
+        <x:v>4.4</x:v>
       </x:c>
       <x:c r="N187" s="26" t="n">
         <x:v>3.3</x:v>
@@ -18091,19 +18158,19 @@
         <x:v>187</x:v>
       </x:c>
       <x:c r="B188" s="20" t="str">
-        <x:v>Justin Watson</x:v>
+        <x:v>Dane Key</x:v>
       </x:c>
       <x:c r="C188" s="16" t="str">
-        <x:v>HOU</x:v>
+        <x:v>DEN</x:v>
       </x:c>
       <x:c r="D188" s="17" t="n">
         <x:v>3.3</x:v>
       </x:c>
       <x:c r="E188" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>2.1</x:v>
       </x:c>
       <x:c r="F188" s="17" t="n">
-        <x:v>25</x:v>
+        <x:v>25.3</x:v>
       </x:c>
       <x:c r="G188" s="17" t="n">
         <x:v>0.1</x:v>
@@ -18121,7 +18188,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L188" s="17" t="n">
-        <x:v>5.3</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="M188" s="17" t="n">
         <x:v>4.3</x:v>
@@ -18135,19 +18202,19 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="B189" s="20" t="str">
-        <x:v>Jake Bobo</x:v>
+        <x:v>Justin Watson</x:v>
       </x:c>
       <x:c r="C189" s="16" t="str">
-        <x:v>SEA</x:v>
+        <x:v>HOU</x:v>
       </x:c>
       <x:c r="D189" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>3.3</x:v>
       </x:c>
       <x:c r="E189" s="17" t="n">
-        <x:v>1.9</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F189" s="17" t="n">
-        <x:v>22.5</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="G189" s="17" t="n">
         <x:v>0.1</x:v>
@@ -18165,13 +18232,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L189" s="17" t="n">
-        <x:v>4.9</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="M189" s="17" t="n">
-        <x:v>3.9</x:v>
+        <x:v>4.3</x:v>
       </x:c>
       <x:c r="N189" s="26" t="n">
-        <x:v>3</x:v>
+        <x:v>3.3</x:v>
       </x:c>
     </x:row>
     <x:row r="190" ht="15" hidden="0" customHeight="1">
@@ -18179,19 +18246,19 @@
         <x:v>189</x:v>
       </x:c>
       <x:c r="B190" s="20" t="str">
-        <x:v>Darius Cooper</x:v>
+        <x:v>Jake Bobo</x:v>
       </x:c>
       <x:c r="C190" s="16" t="str">
-        <x:v>PHI</x:v>
+        <x:v>SEA</x:v>
       </x:c>
       <x:c r="D190" s="17" t="n">
-        <x:v>3.1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E190" s="17" t="n">
         <x:v>1.9</x:v>
       </x:c>
       <x:c r="F190" s="17" t="n">
-        <x:v>20.1</x:v>
+        <x:v>22.5</x:v>
       </x:c>
       <x:c r="G190" s="17" t="n">
         <x:v>0.1</x:v>
@@ -18209,13 +18276,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L190" s="17" t="n">
-        <x:v>4.7</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="M190" s="17" t="n">
-        <x:v>3.8</x:v>
+        <x:v>3.9</x:v>
       </x:c>
       <x:c r="N190" s="26" t="n">
-        <x:v>2.8</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="191" ht="15" hidden="0" customHeight="1">
@@ -21081,7 +21148,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f7d12f3b26645e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R879bf04ddedf4263"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27973,7 +28040,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59fc161d2513432c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5d9201fabf84f6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28017,7 +28084,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B2" s="46" t="str">
-        <x:v>August 12, 2026</x:v>
+        <x:v>August 13, 2026, 2:01 PM ET</x:v>
       </x:c>
       <x:c r="C2" s="46" t="str">
         <x:v>Timezone</x:v>
@@ -29928,139 +29995,542 @@
         <x:v>https://sports.yahoo.com/fantasy/article/nfl-training-camp-injury-report-tracking-the-latest-news-updates-for-2026-fantasy-football-163938278.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="54">
-      <x:c r="A54"/>
-      <x:c r="B54"/>
-      <x:c r="C54"/>
-      <x:c r="D54"/>
-      <x:c r="E54" s="10"/>
-      <x:c r="F54" s="10"/>
-      <x:c r="G54" s="12"/>
-      <x:c r="H54" s="12"/>
-      <x:c r="I54" s="12"/>
-      <x:c r="J54"/>
-      <x:c r="K54"/>
-      <x:c r="L54"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="49" t="str">
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="73" t="str">
+        <x:v>August 13, 2026 incremental update</x:v>
+      </x:c>
+      <x:c r="B54" s="73"/>
+      <x:c r="C54" s="73"/>
+      <x:c r="D54" s="73"/>
+      <x:c r="E54" s="74"/>
+      <x:c r="F54" s="74"/>
+      <x:c r="G54" s="75"/>
+      <x:c r="H54" s="75"/>
+      <x:c r="I54" s="75"/>
+      <x:c r="J54" s="73"/>
+      <x:c r="K54" s="73"/>
+      <x:c r="L54" s="73"/>
+    </x:row>
+    <x:row r="55" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A55" s="92" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="B55" s="92" t="str">
+        <x:v>Chuba Hubbard</x:v>
+      </x:c>
+      <x:c r="C55" s="92" t="str">
+        <x:v>CAR</x:v>
+      </x:c>
+      <x:c r="D55" s="92" t="str">
+        <x:v>UPDATED</x:v>
+      </x:c>
+      <x:c r="E55" s="93" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F55" s="93" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="G55" s="94" t="n">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="H55" s="94" t="n">
+        <x:v>144.9</x:v>
+      </x:c>
+      <x:c r="I55" s="94" t="n">
+        <x:v>-11.1</x:v>
+      </x:c>
+      <x:c r="J55" s="92" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K55" s="92" t="str">
+        <x:v>Hubbard is week-to-week with a legitimate hamstring injury. Carolina remains confident he will be ready for Week 1, so no games were deducted; a modest share of existing backfield opportunity moved to Brooks while team totals stayed unchanged.</x:v>
+      </x:c>
+      <x:c r="L55" s="92" t="str">
+        <x:v>https://www.reuters.com/sports/panthers-rb-chuba-hubbard-hamstring-week-to-week--flm-2026-08-13/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A56" s="92" t="str">
+        <x:v>RB</x:v>
+      </x:c>
+      <x:c r="B56" s="92" t="str">
+        <x:v>Jonathon Brooks</x:v>
+      </x:c>
+      <x:c r="C56" s="92" t="str">
+        <x:v>CAR</x:v>
+      </x:c>
+      <x:c r="D56" s="92" t="str">
+        <x:v>UPDATED</x:v>
+      </x:c>
+      <x:c r="E56" s="93" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F56" s="93" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G56" s="94" t="n">
+        <x:v>131.6</x:v>
+      </x:c>
+      <x:c r="H56" s="94" t="n">
+        <x:v>142.7</x:v>
+      </x:c>
+      <x:c r="I56" s="94" t="n">
+        <x:v>11.1</x:v>
+      </x:c>
+      <x:c r="J56" s="92" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K56" s="92" t="str">
+        <x:v>Hubbard is week-to-week and Brooks is expected to receive significant preseason work. Increased Brooks modestly without adding Carolina team opportunity or assuming Hubbard misses regular-season games.</x:v>
+      </x:c>
+      <x:c r="L56" s="92" t="str">
+        <x:v>https://www.reuters.com/sports/panthers-rb-chuba-hubbard-hamstring-week-to-week--flm-2026-08-13/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A57" s="92" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B57" s="92" t="str">
+        <x:v>Makai Lemon</x:v>
+      </x:c>
+      <x:c r="C57" s="92" t="str">
+        <x:v>PHI</x:v>
+      </x:c>
+      <x:c r="D57" s="92" t="str">
+        <x:v>UPDATED</x:v>
+      </x:c>
+      <x:c r="E57" s="93" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="F57" s="93" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G57" s="94" t="n">
+        <x:v>122.6</x:v>
+      </x:c>
+      <x:c r="H57" s="94" t="n">
+        <x:v>109.2</x:v>
+      </x:c>
+      <x:c r="I57" s="94" t="n">
+        <x:v>-13.4</x:v>
+      </x:c>
+      <x:c r="J57" s="92" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K57" s="92" t="str">
+        <x:v>Lemon continues to miss practice with a hamstring issue after repeated spring and camp absences. Reduced his season-long target share modestly for early-role risk, without projecting missed regular-season games.</x:v>
+      </x:c>
+      <x:c r="L57" s="92" t="str">
+        <x:v>https://www.bleedinggreennation.com/news/179297/cooper-dejean-quinyon-mitchell-added-to-latest-eagles-injury-report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A58" s="92" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B58" s="92" t="str">
+        <x:v>Dontayvion Wicks</x:v>
+      </x:c>
+      <x:c r="C58" s="92" t="str">
+        <x:v>PHI</x:v>
+      </x:c>
+      <x:c r="D58" s="92" t="str">
+        <x:v>RECONCILED</x:v>
+      </x:c>
+      <x:c r="E58" s="93" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="F58" s="93" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="G58" s="94" t="n">
+        <x:v>70.6</x:v>
+      </x:c>
+      <x:c r="H58" s="94" t="n">
+        <x:v>77.1</x:v>
+      </x:c>
+      <x:c r="I58" s="94" t="n">
+        <x:v>6.5</x:v>
+      </x:c>
+      <x:c r="J58" s="92" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K58" s="92" t="str">
+        <x:v>Lemon's modest target reduction was redistributed within the Eagles receiver room. Wicks received the largest share because he has already taken advantage of additional camp reps.</x:v>
+      </x:c>
+      <x:c r="L58" s="92" t="str">
+        <x:v>https://www.bleedinggreennation.com/news/179297/cooper-dejean-quinyon-mitchell-added-to-latest-eagles-injury-report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A59" s="92" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B59" s="92" t="str">
+        <x:v>Hollywood Brown</x:v>
+      </x:c>
+      <x:c r="C59" s="92" t="str">
+        <x:v>PHI</x:v>
+      </x:c>
+      <x:c r="D59" s="92" t="str">
+        <x:v>RECONCILED</x:v>
+      </x:c>
+      <x:c r="E59" s="93" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F59" s="93" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G59" s="94" t="n">
+        <x:v>64.5</x:v>
+      </x:c>
+      <x:c r="H59" s="94" t="n">
+        <x:v>67.8</x:v>
+      </x:c>
+      <x:c r="I59" s="94" t="n">
+        <x:v>3.3</x:v>
+      </x:c>
+      <x:c r="J59" s="92" t="str">
+        <x:v>Medium-Low</x:v>
+      </x:c>
+      <x:c r="K59" s="92" t="str">
+        <x:v>Received a small share of the Eagles targets removed from Lemon. No independent breakout adjustment was applied.</x:v>
+      </x:c>
+      <x:c r="L59" s="92" t="str">
+        <x:v>https://www.bleedinggreennation.com/news/179297/cooper-dejean-quinyon-mitchell-added-to-latest-eagles-injury-report</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A60" s="92" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B60" s="92" t="str">
+        <x:v>Darius Cooper</x:v>
+      </x:c>
+      <x:c r="C60" s="92" t="str">
+        <x:v>PHI</x:v>
+      </x:c>
+      <x:c r="D60" s="92" t="str">
+        <x:v>RECONCILED</x:v>
+      </x:c>
+      <x:c r="E60" s="93" t="n">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="F60" s="93" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="G60" s="94" t="n">
+        <x:v>4.7</x:v>
+      </x:c>
+      <x:c r="H60" s="94" t="n">
+        <x:v>7.8</x:v>
+      </x:c>
+      <x:c r="I60" s="94" t="n">
+        <x:v>3.1</x:v>
+      </x:c>
+      <x:c r="J60" s="92" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K60" s="92" t="str">
+        <x:v>Received a small share of the Eagles targets removed from Lemon. Cooper has continued to impress in camp and Nick Sirianni acknowledged the possibility of offensive playing time.</x:v>
+      </x:c>
+      <x:c r="L60" s="92" t="str">
+        <x:v>https://www.bleedinggreennation.com/philadelphia-eagles-preseason/179299/eagles-training-camp-notes-practice-ends-after-a-fight-breaks-out</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A61" s="92" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B61" s="92" t="str">
+        <x:v>Emeka Egbuka</x:v>
+      </x:c>
+      <x:c r="C61" s="92" t="str">
+        <x:v>TB</x:v>
+      </x:c>
+      <x:c r="D61" s="92" t="str">
+        <x:v>WATCH, NO CHANGE</x:v>
+      </x:c>
+      <x:c r="E61" s="92" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F61" s="92" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G61" s="92" t="n">
+        <x:v>211.9</x:v>
+      </x:c>
+      <x:c r="H61" s="92" t="n">
+        <x:v>211.9</x:v>
+      </x:c>
+      <x:c r="I61" s="92" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J61" s="92" t="str">
+        <x:v>Uncertain</x:v>
+      </x:c>
+      <x:c r="K61" s="92" t="str">
+        <x:v>Toe injury may cost preseason time, but the exact severity and regular-season impact are not established. No games or targets deducted yet.</x:v>
+      </x:c>
+      <x:c r="L61" s="92" t="str">
+        <x:v>https://www.bucsnation.com/tampa-bay-buccaneers-news/68109/tampa-bay-buccaneers-news-emeka-egbuka-injury-update-sparks-concern</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A62" s="92" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B62" s="92" t="str">
+        <x:v>Malik Nabers</x:v>
+      </x:c>
+      <x:c r="C62" s="92" t="str">
+        <x:v>NYG</x:v>
+      </x:c>
+      <x:c r="D62" s="92" t="str">
+        <x:v>WATCH, NO CHANGE</x:v>
+      </x:c>
+      <x:c r="E62" s="92" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F62" s="92" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="G62" s="92" t="n">
+        <x:v>202.5</x:v>
+      </x:c>
+      <x:c r="H62" s="92" t="n">
+        <x:v>202.5</x:v>
+      </x:c>
+      <x:c r="I62" s="92" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J62" s="92" t="str">
+        <x:v>Medium-Low</x:v>
+      </x:c>
+      <x:c r="K62" s="92" t="str">
+        <x:v>Rehab is progressing and he could begin 7-on-7/11-on-11 work soon, but he has not yet completed full team work. Current recovery discount remains unchanged.</x:v>
+      </x:c>
+      <x:c r="L62" s="92" t="str">
+        <x:v>https://nypost.com/2026/08/12/sports/malik-nabers-could-take-next-big-giants-rehab-step-on-monday/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A63" s="92" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="B63" s="92" t="str">
+        <x:v>Deshaun Watson</x:v>
+      </x:c>
+      <x:c r="C63" s="92" t="str">
+        <x:v>CLE</x:v>
+      </x:c>
+      <x:c r="D63" s="92" t="str">
+        <x:v>WATCH, NO CHANGE</x:v>
+      </x:c>
+      <x:c r="E63" s="92" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F63" s="92" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="G63" s="92" t="n">
+        <x:v>107.4</x:v>
+      </x:c>
+      <x:c r="H63" s="92" t="n">
+        <x:v>107.4</x:v>
+      </x:c>
+      <x:c r="I63" s="92" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J63" s="92" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K63" s="92" t="str">
+        <x:v>Watson will start preseason Game 1, while Sanders will start Game 2. Todd Monken says the competition remains open, so Cleveland's existing QB allocation is unchanged.</x:v>
+      </x:c>
+      <x:c r="L63" s="92" t="str">
+        <x:v>https://www.reuters.com/sports/browns-will-start-qb-deshaun-watson-preseason-opener-vs-bears--flm-2026-08-12/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A64" s="92" t="str">
+        <x:v>QB</x:v>
+      </x:c>
+      <x:c r="B64" s="92" t="str">
+        <x:v>Shedeur Sanders</x:v>
+      </x:c>
+      <x:c r="C64" s="92" t="str">
+        <x:v>CLE</x:v>
+      </x:c>
+      <x:c r="D64" s="92" t="str">
+        <x:v>WATCH, NO CHANGE</x:v>
+      </x:c>
+      <x:c r="E64" s="92" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F64" s="92" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G64" s="92" t="n">
+        <x:v>115.1</x:v>
+      </x:c>
+      <x:c r="H64" s="92" t="n">
+        <x:v>115.1</x:v>
+      </x:c>
+      <x:c r="I64" s="92" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J64" s="92" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="K64" s="92" t="str">
+        <x:v>Sanders will start preseason Game 2 after Watson starts Game 1. The coach says the competition remains open, so Cleveland's existing QB allocation is unchanged.</x:v>
+      </x:c>
+      <x:c r="L64" s="92" t="str">
+        <x:v>https://www.reuters.com/sports/browns-will-start-qb-deshaun-watson-preseason-opener-vs-bears--flm-2026-08-12/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
         <x:v>Validation</x:v>
       </x:c>
-      <x:c r="B55" s="49" t="str"/>
-      <x:c r="C55" s="49" t="str"/>
-      <x:c r="D55" s="49" t="str"/>
-      <x:c r="E55" s="65" t="str"/>
-      <x:c r="F55" s="65" t="str"/>
-      <x:c r="G55" s="59" t="str"/>
-      <x:c r="H55" s="59" t="str"/>
-      <x:c r="I55" s="59" t="str"/>
-      <x:c r="J55" s="49" t="str"/>
-      <x:c r="K55" s="49" t="str"/>
-      <x:c r="L55" s="49" t="str"/>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="54" t="str">
+      <x:c r="B66"/>
+      <x:c r="C66"/>
+      <x:c r="D66"/>
+      <x:c r="E66"/>
+      <x:c r="F66"/>
+      <x:c r="G66"/>
+      <x:c r="H66"/>
+      <x:c r="I66"/>
+      <x:c r="J66"/>
+      <x:c r="K66"/>
+      <x:c r="L66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
         <x:v>Check</x:v>
       </x:c>
-      <x:c r="B56" s="54" t="str">
+      <x:c r="B67" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="C56" s="54" t="str">
+      <x:c r="C67" t="str">
         <x:v>Details</x:v>
       </x:c>
-      <x:c r="D56" s="54" t="str"/>
-      <x:c r="E56" s="66" t="str"/>
-      <x:c r="F56" s="66" t="str"/>
-      <x:c r="G56" s="60" t="str"/>
-      <x:c r="H56" s="60" t="str"/>
-      <x:c r="I56" s="60" t="str"/>
-      <x:c r="J56" s="54" t="str"/>
-      <x:c r="K56" s="54" t="str"/>
-      <x:c r="L56" s="54" t="str"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="45" t="str">
+      <x:c r="D67"/>
+      <x:c r="E67"/>
+      <x:c r="F67"/>
+      <x:c r="G67"/>
+      <x:c r="H67"/>
+      <x:c r="I67"/>
+      <x:c r="J67"/>
+      <x:c r="K67"/>
+      <x:c r="L67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
         <x:v>Negative projected stats</x:v>
       </x:c>
-      <x:c r="B57" s="45" t="str">
+      <x:c r="B68" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="C57" s="45" t="str">
+      <x:c r="C68" t="str">
         <x:v>No negative projected stat values remain in QB/RB/WR/TE sheets.</x:v>
       </x:c>
-      <x:c r="D57" s="45" t="str"/>
-      <x:c r="E57" s="62" t="str"/>
-      <x:c r="F57" s="62" t="str"/>
-      <x:c r="G57" s="56" t="str"/>
-      <x:c r="H57" s="56" t="str"/>
-      <x:c r="I57" s="56" t="str"/>
-      <x:c r="J57" s="45" t="str"/>
-      <x:c r="K57" s="45" t="str"/>
-      <x:c r="L57" s="45" t="str"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="45" t="str">
+      <x:c r="D68"/>
+      <x:c r="E68"/>
+      <x:c r="F68"/>
+      <x:c r="G68"/>
+      <x:c r="H68"/>
+      <x:c r="I68"/>
+      <x:c r="J68"/>
+      <x:c r="K68"/>
+      <x:c r="L68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
         <x:v>Receptions &gt; targets</x:v>
       </x:c>
-      <x:c r="B58" s="45" t="str">
+      <x:c r="B69" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="C58" s="45" t="str">
+      <x:c r="C69" t="str">
         <x:v>No player has receptions greater than targets.</x:v>
       </x:c>
-      <x:c r="D58" s="45" t="str"/>
-      <x:c r="E58" s="62" t="str"/>
-      <x:c r="F58" s="62" t="str"/>
-      <x:c r="G58" s="56" t="str"/>
-      <x:c r="H58" s="56" t="str"/>
-      <x:c r="I58" s="56" t="str"/>
-      <x:c r="J58" s="45" t="str"/>
-      <x:c r="K58" s="45" t="str"/>
-      <x:c r="L58" s="45" t="str"/>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="45" t="str">
+      <x:c r="D69"/>
+      <x:c r="E69"/>
+      <x:c r="F69"/>
+      <x:c r="G69"/>
+      <x:c r="H69"/>
+      <x:c r="I69"/>
+      <x:c r="J69"/>
+      <x:c r="K69"/>
+      <x:c r="L69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
         <x:v>Affected receiving team totals</x:v>
       </x:c>
-      <x:c r="B59" s="45" t="str">
+      <x:c r="B70" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="C59" s="45" t="str">
-        <x:v>Targets, receptions, receiving yards and receiving TDs were preserved for SF, CAR, GB, CLE, MIA, SEA, DAL, NYG and JAX.</x:v>
-      </x:c>
-      <x:c r="D59" s="45" t="str"/>
-      <x:c r="E59" s="62" t="str"/>
-      <x:c r="F59" s="62" t="str"/>
-      <x:c r="G59" s="56" t="str"/>
-      <x:c r="H59" s="56" t="str"/>
-      <x:c r="I59" s="56" t="str"/>
-      <x:c r="J59" s="45" t="str"/>
-      <x:c r="K59" s="45" t="str"/>
-      <x:c r="L59" s="45" t="str"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="45" t="str">
+      <x:c r="C70" t="str">
+        <x:v>Targets, receptions, receiving yards and receiving TDs remain preserved for prior reconciled teams and for Philadelphia in the August 13 update.</x:v>
+      </x:c>
+      <x:c r="D70"/>
+      <x:c r="E70"/>
+      <x:c r="F70"/>
+      <x:c r="G70"/>
+      <x:c r="H70"/>
+      <x:c r="I70"/>
+      <x:c r="J70"/>
+      <x:c r="K70"/>
+      <x:c r="L70"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
         <x:v>Starter-reallocation team totals</x:v>
       </x:c>
-      <x:c r="B60" s="45" t="str">
+      <x:c r="B71" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="C60" s="45" t="str">
-        <x:v>Minnesota and Las Vegas aggregate QB passing and rushing budgets were preserved exactly while starter shares changed.</x:v>
-      </x:c>
-      <x:c r="D60" s="45" t="str"/>
-      <x:c r="E60" s="62" t="str"/>
-      <x:c r="F60" s="62" t="str"/>
-      <x:c r="G60" s="56" t="str"/>
-      <x:c r="H60" s="56" t="str"/>
-      <x:c r="I60" s="56" t="str"/>
-      <x:c r="J60" s="45" t="str"/>
-      <x:c r="K60" s="45" t="str"/>
-      <x:c r="L60" s="45" t="str"/>
+      <x:c r="C71" t="str">
+        <x:v>Minnesota and Las Vegas aggregate QB passing and rushing budgets remain preserved exactly while starter shares changed.</x:v>
+      </x:c>
+      <x:c r="D71"/>
+      <x:c r="E71"/>
+      <x:c r="F71"/>
+      <x:c r="G71"/>
+      <x:c r="H71"/>
+      <x:c r="I71"/>
+      <x:c r="J71"/>
+      <x:c r="K71"/>
+      <x:c r="L71"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>Carolina backfield totals</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Carolina RB targets, receptions, receiving yards/TDs, rush attempts, rushing yards/TDs and fumbles lost are unchanged; opportunity was only reallocated between Hubbard and Brooks.</x:v>
+      </x:c>
+      <x:c r="D72"/>
+      <x:c r="E72"/>
+      <x:c r="F72"/>
+      <x:c r="G72"/>
+      <x:c r="H72"/>
+      <x:c r="I72"/>
+      <x:c r="J72"/>
+      <x:c r="K72"/>
+      <x:c r="L72"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A54:L54"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Refresh NFL projections rankings and ADP
</commit_message>
<xml_diff>
--- a/data/projections.xlsx
+++ b/data/projections.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QB" sheetId="1" r:id="R2a696b901a2c40b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="2" r:id="Rd38ac66a6b174ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WR" sheetId="3" r:id="Rc46ecbfbe24f493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TE" sheetId="4" r:id="R9835e52518b8415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Update" sheetId="5" r:id="R24a4ed4641cb4d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QB" sheetId="1" r:id="R7d43bf37c6254be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="2" r:id="Rdf682e3a2cba453a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WR" sheetId="3" r:id="R7593fea4eea94747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TE" sheetId="4" r:id="R9ca4e15c1c1646d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Update" sheetId="5" r:id="R6281eb41920041b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2599,7 +2599,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1488efdaa88246e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44035cbc9ecb426f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10091,7 +10091,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bf03de1462243f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf335419fd37e4d05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10366,7 +10366,7 @@
     </x:row>
     <x:row r="6" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A6" s="99" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
         <x:v>Justin Jefferson</x:v>
@@ -10410,7 +10410,7 @@
     </x:row>
     <x:row r="7" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A7" s="99" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="20" t="str">
         <x:v>Nico Collins</x:v>
@@ -10586,7 +10586,7 @@
     </x:row>
     <x:row r="11" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A11" s="99" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B11" s="20" t="str">
         <x:v>Chris Olave</x:v>
@@ -10630,7 +10630,7 @@
     </x:row>
     <x:row r="12" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A12" s="99" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="20" t="str">
         <x:v>A.J. Brown</x:v>
@@ -10806,7 +10806,7 @@
     </x:row>
     <x:row r="16" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A16" s="99" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B16" s="20" t="str">
         <x:v>DeVonta Smith</x:v>
@@ -10850,7 +10850,7 @@
     </x:row>
     <x:row r="17" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A17" s="99" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B17" s="20" t="str">
         <x:v>Garrett Wilson</x:v>
@@ -10894,7 +10894,7 @@
     </x:row>
     <x:row r="18" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A18" s="99" t="n">
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B18" s="20" t="str">
         <x:v>Tee Higgins</x:v>
@@ -10938,7 +10938,7 @@
     </x:row>
     <x:row r="19" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A19" s="99" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B19" s="20" t="str">
         <x:v>Marvin Harrison Jr.</x:v>
@@ -11070,7 +11070,7 @@
     </x:row>
     <x:row r="22" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A22" s="99" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B22" s="20" t="str">
         <x:v>Luther Burden III</x:v>
@@ -11114,7 +11114,7 @@
     </x:row>
     <x:row r="23" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A23" s="99" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B23" s="20" t="str">
         <x:v>DJ Moore</x:v>
@@ -11158,7 +11158,7 @@
     </x:row>
     <x:row r="24" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A24" s="99" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B24" s="20" t="str">
         <x:v>Terry McLaurin</x:v>
@@ -11202,7 +11202,7 @@
     </x:row>
     <x:row r="25" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A25" s="99" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B25" s="20" t="str">
         <x:v>Malik Nabers</x:v>
@@ -11246,7 +11246,7 @@
     </x:row>
     <x:row r="26" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A26" s="99" t="n">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="20" t="str">
         <x:v>Jameson Williams</x:v>
@@ -11334,7 +11334,7 @@
     </x:row>
     <x:row r="28" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A28" s="99" t="n">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B28" s="20" t="str">
         <x:v>Ladd McConkey</x:v>
@@ -11378,7 +11378,7 @@
     </x:row>
     <x:row r="29" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A29" s="99" t="n">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B29" s="20" t="str">
         <x:v>Mike Evans</x:v>
@@ -11422,7 +11422,7 @@
     </x:row>
     <x:row r="30" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A30" s="99" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B30" s="20" t="str">
         <x:v>Courtland Sutton</x:v>
@@ -11466,7 +11466,7 @@
     </x:row>
     <x:row r="31" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A31" s="99" t="n">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B31" s="20" t="str">
         <x:v>Wan'Dale Robinson</x:v>
@@ -11510,7 +11510,7 @@
     </x:row>
     <x:row r="32" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A32" s="99" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B32" s="20" t="str">
         <x:v>Davante Adams</x:v>
@@ -11554,7 +11554,7 @@
     </x:row>
     <x:row r="33" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A33" s="99" t="n">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B33" s="20" t="str">
         <x:v>DK Metcalf</x:v>
@@ -11598,7 +11598,7 @@
     </x:row>
     <x:row r="34" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A34" s="99" t="n">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B34" s="20" t="str">
         <x:v>Christian Watson</x:v>
@@ -11642,7 +11642,7 @@
     </x:row>
     <x:row r="35" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A35" s="99" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B35" s="20" t="str">
         <x:v>Michael Wilson</x:v>
@@ -11686,7 +11686,7 @@
     </x:row>
     <x:row r="36" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A36" s="99" t="n">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B36" s="20" t="str">
         <x:v>Michael Pittman Jr.</x:v>
@@ -11730,7 +11730,7 @@
     </x:row>
     <x:row r="37" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A37" s="99" t="n">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
         <x:v>Parker Washington</x:v>
@@ -11774,7 +11774,7 @@
     </x:row>
     <x:row r="38" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A38" s="99" t="n">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
         <x:v>Brian Thomas Jr.</x:v>
@@ -11862,7 +11862,7 @@
     </x:row>
     <x:row r="40" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A40" s="99" t="n">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B40" s="20" t="str">
         <x:v>Matthew Golden</x:v>
@@ -11906,7 +11906,7 @@
     </x:row>
     <x:row r="41" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A41" s="99" t="n">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B41" s="20" t="str">
         <x:v>Jordan Addison</x:v>
@@ -11950,7 +11950,7 @@
     </x:row>
     <x:row r="42" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A42" s="99" t="n">
-        <x:v>41</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B42" s="20" t="str">
         <x:v>Alec Pierce</x:v>
@@ -12038,7 +12038,7 @@
     </x:row>
     <x:row r="44" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A44" s="99" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B44" s="20" t="str">
         <x:v>Josh Downs</x:v>
@@ -12082,7 +12082,7 @@
     </x:row>
     <x:row r="45" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A45" s="99" t="n">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B45" s="20" t="str">
         <x:v>Stefon Diggs</x:v>
@@ -12126,7 +12126,7 @@
     </x:row>
     <x:row r="46" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A46" s="99" t="n">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B46" s="20" t="str">
         <x:v>Tre Tucker</x:v>
@@ -12170,7 +12170,7 @@
     </x:row>
     <x:row r="47" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A47" s="99" t="n">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B47" s="20" t="str">
         <x:v>Xavier Worthy</x:v>
@@ -12258,7 +12258,7 @@
     </x:row>
     <x:row r="49" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A49" s="99" t="n">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B49" s="20" t="str">
         <x:v>Chris Godwin Jr.</x:v>
@@ -12302,7 +12302,7 @@
     </x:row>
     <x:row r="50" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A50" s="99" t="n">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B50" s="20" t="str">
         <x:v>Adonai Mitchell</x:v>
@@ -12346,7 +12346,7 @@
     </x:row>
     <x:row r="51" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A51" s="99" t="n">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B51" s="20" t="str">
         <x:v>Carnell Tate</x:v>
@@ -12390,7 +12390,7 @@
     </x:row>
     <x:row r="52" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A52" s="99" t="n">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B52" s="20" t="str">
         <x:v>Khalil Shakir</x:v>
@@ -12478,7 +12478,7 @@
     </x:row>
     <x:row r="54" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A54" s="99" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B54" s="20" t="str">
         <x:v>Denzel Boston</x:v>
@@ -12522,7 +12522,7 @@
     </x:row>
     <x:row r="55" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A55" s="99" t="n">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B55" s="20" t="str">
         <x:v>Rashid Shaheed</x:v>
@@ -12654,7 +12654,7 @@
     </x:row>
     <x:row r="58" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A58" s="99" t="n">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B58" s="20" t="str">
         <x:v>Keenan Allen</x:v>
@@ -12698,7 +12698,7 @@
     </x:row>
     <x:row r="59" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A59" s="99" t="n">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B59" s="20" t="str">
         <x:v>Tank Dell</x:v>
@@ -12742,7 +12742,7 @@
     </x:row>
     <x:row r="60" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A60" s="99" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B60" s="20" t="str">
         <x:v>KC Concepcion</x:v>
@@ -12786,7 +12786,7 @@
     </x:row>
     <x:row r="61" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A61" s="99" t="n">
-        <x:v>60</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B61" s="20" t="str">
         <x:v>Calvin Ridley</x:v>
@@ -12918,7 +12918,7 @@
     </x:row>
     <x:row r="64" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A64" s="99" t="n">
-        <x:v>63</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B64" s="20" t="str">
         <x:v>John Metchie III</x:v>
@@ -12962,7 +12962,7 @@
     </x:row>
     <x:row r="65" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A65" s="99" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B65" s="20" t="str">
         <x:v>Zachariah Branch</x:v>
@@ -13006,7 +13006,7 @@
     </x:row>
     <x:row r="66" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A66" s="99" t="n">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B66" s="20" t="str">
         <x:v>Deebo Samuel Sr.</x:v>
@@ -13050,7 +13050,7 @@
     </x:row>
     <x:row r="67" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A67" s="99" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B67" s="20" t="str">
         <x:v>Jalen Coker</x:v>
@@ -13094,7 +13094,7 @@
     </x:row>
     <x:row r="68" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A68" s="99" t="n">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B68" s="20" t="str">
         <x:v>Romeo Doubs</x:v>
@@ -13138,7 +13138,7 @@
     </x:row>
     <x:row r="69" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A69" s="99" t="n">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B69" s="20" t="str">
         <x:v>Omar Cooper Jr.</x:v>
@@ -13182,7 +13182,7 @@
     </x:row>
     <x:row r="70" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A70" s="99" t="n">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B70" s="20" t="str">
         <x:v>Jalen McMillan</x:v>
@@ -13226,7 +13226,7 @@
     </x:row>
     <x:row r="71" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A71" s="99" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B71" s="20" t="str">
         <x:v>Andrei Iosivas</x:v>
@@ -13270,7 +13270,7 @@
     </x:row>
     <x:row r="72" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A72" s="99" t="n">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B72" s="20" t="str">
         <x:v>Rashod Bateman</x:v>
@@ -13314,7 +13314,7 @@
     </x:row>
     <x:row r="73" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A73" s="99" t="n">
-        <x:v>72</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B73" s="20" t="str">
         <x:v>Malik Washington</x:v>
@@ -13358,7 +13358,7 @@
     </x:row>
     <x:row r="74" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A74" s="99" t="n">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B74" s="20" t="str">
         <x:v>Ted Hurst</x:v>
@@ -13402,7 +13402,7 @@
     </x:row>
     <x:row r="75" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A75" s="99" t="n">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B75" s="20" t="str">
         <x:v>Theo Wease Jr.</x:v>
@@ -13490,7 +13490,7 @@
     </x:row>
     <x:row r="77" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A77" s="99" t="n">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B77" s="20" t="str">
         <x:v>Troy Franklin</x:v>
@@ -13534,7 +13534,7 @@
     </x:row>
     <x:row r="78" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A78" s="99" t="n">
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B78" s="20" t="str">
         <x:v>Malik Benson</x:v>
@@ -13578,7 +13578,7 @@
     </x:row>
     <x:row r="79" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A79" s="99" t="n">
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B79" s="20" t="str">
         <x:v>Christian Kirk</x:v>
@@ -13622,7 +13622,7 @@
     </x:row>
     <x:row r="80" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A80" s="99" t="n">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B80" s="20" t="str">
         <x:v>Isaac TeSlaa</x:v>
@@ -13666,7 +13666,7 @@
     </x:row>
     <x:row r="81" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A81" s="99" t="n">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B81" s="20" t="str">
         <x:v>Ja'Kobi Lane</x:v>
@@ -13710,7 +13710,7 @@
     </x:row>
     <x:row r="82" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A82" s="99" t="n">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B82" s="20" t="str">
         <x:v>Jaylin Noel</x:v>
@@ -13754,7 +13754,7 @@
     </x:row>
     <x:row r="83" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A83" s="99" t="n">
-        <x:v>82</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B83" s="20" t="str">
         <x:v>Dontayvion Wicks</x:v>
@@ -13798,7 +13798,7 @@
     </x:row>
     <x:row r="84" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A84" s="99" t="n">
-        <x:v>83</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B84" s="20" t="str">
         <x:v>Jack Bech</x:v>
@@ -13842,7 +13842,7 @@
     </x:row>
     <x:row r="85" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A85" s="99" t="n">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B85" s="20" t="str">
         <x:v>Cooper Kupp</x:v>
@@ -13886,7 +13886,7 @@
     </x:row>
     <x:row r="86" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A86" s="99" t="n">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B86" s="20" t="str">
         <x:v>De'Zhaun Stribling</x:v>
@@ -13930,7 +13930,7 @@
     </x:row>
     <x:row r="87" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A87" s="99" t="n">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B87" s="20" t="str">
         <x:v>Jordyn Tyson</x:v>
@@ -13974,13 +13974,13 @@
     </x:row>
     <x:row r="88" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A88" s="99" t="n">
-        <x:v>87</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B88" s="20" t="str">
         <x:v>Kayshon Boutte</x:v>
       </x:c>
       <x:c r="C88" s="16" t="str">
-        <x:v>NE</x:v>
+        <x:v>HOU</x:v>
       </x:c>
       <x:c r="D88" s="100" t="n">
         <x:v>33.7</x:v>
@@ -14018,7 +14018,7 @@
     </x:row>
     <x:row r="89" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A89" s="99" t="n">
-        <x:v>88</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B89" s="20" t="str">
         <x:v>Tyquan Thornton</x:v>
@@ -14106,7 +14106,7 @@
     </x:row>
     <x:row r="91" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A91" s="99" t="n">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B91" s="20" t="str">
         <x:v>Caleb Douglas</x:v>
@@ -14194,7 +14194,7 @@
     </x:row>
     <x:row r="93" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A93" s="99" t="n">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B93" s="20" t="str">
         <x:v>Elic Ayomanor</x:v>
@@ -14238,25 +14238,25 @@
     </x:row>
     <x:row r="94" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A94" s="99" t="n">
-        <x:v>93</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="B94" s="20" t="str">
         <x:v>Cedric Tillman</x:v>
       </x:c>
       <x:c r="C94" s="16" t="str">
-        <x:v>CLE</x:v>
+        <x:v>FA</x:v>
       </x:c>
       <x:c r="D94" s="100" t="n">
-        <x:v>43.2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E94" s="100" t="n">
-        <x:v>24.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F94" s="100" t="n">
-        <x:v>301.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G94" s="100" t="n">
-        <x:v>2.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H94" s="100" t="n">
         <x:v>0</x:v>
@@ -14271,18 +14271,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L94" s="100" t="n">
-        <x:v>68.8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M94" s="100" t="n">
-        <x:v>56.4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N94" s="101" t="n">
-        <x:v>43.9</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O94" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="95" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A95" s="99" t="n">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B95" s="20" t="str">
         <x:v>Hollywood Brown</x:v>
@@ -14326,7 +14329,7 @@
     </x:row>
     <x:row r="96" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A96" s="99" t="n">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B96" s="20" t="str">
         <x:v>Mack Hollins</x:v>
@@ -14370,7 +14373,7 @@
     </x:row>
     <x:row r="97" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A97" s="99" t="n">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B97" s="20" t="str">
         <x:v>Travis Hunter</x:v>
@@ -14414,7 +14417,7 @@
     </x:row>
     <x:row r="98" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A98" s="99" t="n">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B98" s="20" t="str">
         <x:v>Joshua Palmer</x:v>
@@ -14458,7 +14461,7 @@
     </x:row>
     <x:row r="99" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A99" s="99" t="n">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B99" s="20" t="str">
         <x:v>Jalen Tolbert</x:v>
@@ -14502,7 +14505,7 @@
     </x:row>
     <x:row r="100" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A100" s="99" t="n">
-        <x:v>99</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B100" s="20" t="str">
         <x:v>Xavier Hutchinson</x:v>
@@ -14546,7 +14549,7 @@
     </x:row>
     <x:row r="101" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A101" s="99" t="n">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B101" s="20" t="str">
         <x:v>Chimere Dike</x:v>
@@ -14634,7 +14637,7 @@
     </x:row>
     <x:row r="103" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A103" s="99" t="n">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B103" s="20" t="str">
         <x:v>Xavier Legette</x:v>
@@ -14678,7 +14681,7 @@
     </x:row>
     <x:row r="104" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A104" s="99" t="n">
-        <x:v>103</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B104" s="20" t="str">
         <x:v>Pat Bryant</x:v>
@@ -14766,7 +14769,7 @@
     </x:row>
     <x:row r="106" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A106" s="99" t="n">
-        <x:v>105</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B106" s="20" t="str">
         <x:v>Jahdae Walker</x:v>
@@ -14810,7 +14813,7 @@
     </x:row>
     <x:row r="107" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A107" s="99" t="n">
-        <x:v>106</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B107" s="20" t="str">
         <x:v>Elijah Sarratt</x:v>
@@ -14854,7 +14857,7 @@
     </x:row>
     <x:row r="108" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A108" s="99" t="n">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B108" s="20" t="str">
         <x:v>Keon Coleman</x:v>
@@ -14898,7 +14901,7 @@
     </x:row>
     <x:row r="109" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A109" s="99" t="n">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B109" s="20" t="str">
         <x:v>Kendrick Bourne</x:v>
@@ -14942,7 +14945,7 @@
     </x:row>
     <x:row r="110" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A110" s="99" t="n">
-        <x:v>109</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B110" s="20" t="str">
         <x:v>Jahan Dotson</x:v>
@@ -14986,7 +14989,7 @@
     </x:row>
     <x:row r="111" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A111" s="99" t="n">
-        <x:v>110</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B111" s="20" t="str">
         <x:v>Olamide Zaccheaus</x:v>
@@ -15030,7 +15033,7 @@
     </x:row>
     <x:row r="112" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A112" s="99" t="n">
-        <x:v>111</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B112" s="20" t="str">
         <x:v>Savion Williams</x:v>
@@ -15074,7 +15077,7 @@
     </x:row>
     <x:row r="113" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A113" s="99" t="n">
-        <x:v>112</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B113" s="20" t="str">
         <x:v>Darnell Mooney</x:v>
@@ -15118,7 +15121,7 @@
     </x:row>
     <x:row r="114" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A114" s="99" t="n">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B114" s="20" t="str">
         <x:v>Devaughn Vele</x:v>
@@ -15162,7 +15165,7 @@
     </x:row>
     <x:row r="115" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A115" s="99" t="n">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B115" s="20" t="str">
         <x:v>Malachi Fields</x:v>
@@ -15206,7 +15209,7 @@
     </x:row>
     <x:row r="116" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A116" s="99" t="n">
-        <x:v>115</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B116" s="20" t="str">
         <x:v>Tory Horton</x:v>
@@ -15250,7 +15253,7 @@
     </x:row>
     <x:row r="117" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A117" s="99" t="n">
-        <x:v>116</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B117" s="20" t="str">
         <x:v>Marvin Mims Jr.</x:v>
@@ -15294,7 +15297,7 @@
     </x:row>
     <x:row r="118" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A118" s="99" t="n">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B118" s="20" t="str">
         <x:v>Bub Means</x:v>
@@ -15382,7 +15385,7 @@
     </x:row>
     <x:row r="120" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A120" s="99" t="n">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B120" s="20" t="str">
         <x:v>Cyrus Allen</x:v>
@@ -15426,7 +15429,7 @@
     </x:row>
     <x:row r="121" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A121" s="99" t="n">
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B121" s="20" t="str">
         <x:v>Kyle Williams</x:v>
@@ -15470,7 +15473,7 @@
     </x:row>
     <x:row r="122" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A122" s="99" t="n">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B122" s="20" t="str">
         <x:v>DeMario Douglas</x:v>
@@ -15602,7 +15605,7 @@
     </x:row>
     <x:row r="125" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A125" s="99" t="n">
-        <x:v>124</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B125" s="20" t="str">
         <x:v>KaVontae Turpin</x:v>
@@ -15646,7 +15649,7 @@
     </x:row>
     <x:row r="126" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A126" s="99" t="n">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B126" s="20" t="str">
         <x:v>Calvin Austin III</x:v>
@@ -15822,7 +15825,7 @@
     </x:row>
     <x:row r="130" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A130" s="99" t="n">
-        <x:v>129</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B130" s="20" t="str">
         <x:v>Ashton Dulin</x:v>
@@ -15910,7 +15913,7 @@
     </x:row>
     <x:row r="132" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A132" s="99" t="n">
-        <x:v>131</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B132" s="20" t="str">
         <x:v>Dyami Brown</x:v>
@@ -15954,13 +15957,13 @@
     </x:row>
     <x:row r="133" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A133" s="99" t="n">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B133" s="20" t="str">
         <x:v>Tutu Atwell</x:v>
       </x:c>
       <x:c r="C133" s="16" t="str">
-        <x:v>MIA</x:v>
+        <x:v>LAR</x:v>
       </x:c>
       <x:c r="D133" s="100" t="n">
         <x:v>21.2</x:v>
@@ -15998,7 +16001,7 @@
     </x:row>
     <x:row r="134" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A134" s="99" t="n">
-        <x:v>133</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B134" s="20" t="str">
         <x:v>Odell Beckham Jr.</x:v>
@@ -16042,7 +16045,7 @@
     </x:row>
     <x:row r="135" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A135" s="99" t="n">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B135" s="20" t="str">
         <x:v>Kevin Coleman Jr.</x:v>
@@ -16086,7 +16089,7 @@
     </x:row>
     <x:row r="136" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A136" s="99" t="n">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B136" s="20" t="str">
         <x:v>Demarcus Robinson</x:v>
@@ -16130,7 +16133,7 @@
     </x:row>
     <x:row r="137" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A137" s="99" t="n">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B137" s="20" t="str">
         <x:v>Van Jefferson</x:v>
@@ -16174,7 +16177,7 @@
     </x:row>
     <x:row r="138" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A138" s="99" t="n">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B138" s="20" t="str">
         <x:v>Nick Westbrook-Ikhine</x:v>
@@ -16218,7 +16221,7 @@
     </x:row>
     <x:row r="139" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A139" s="99" t="n">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B139" s="20" t="str">
         <x:v>Treylon Burks</x:v>
@@ -16262,7 +16265,7 @@
     </x:row>
     <x:row r="140" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A140" s="99" t="n">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B140" s="20" t="str">
         <x:v>Zavion Thomas</x:v>
@@ -16306,7 +16309,7 @@
     </x:row>
     <x:row r="141" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A141" s="99" t="n">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B141" s="20" t="str">
         <x:v>Jaylin Lane</x:v>
@@ -16350,7 +16353,7 @@
     </x:row>
     <x:row r="142" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A142" s="99" t="n">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B142" s="20" t="str">
         <x:v>Dont'e Thornton Jr.</x:v>
@@ -16394,7 +16397,7 @@
     </x:row>
     <x:row r="143" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A143" s="99" t="n">
-        <x:v>142</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B143" s="20" t="str">
         <x:v>Tim Patrick</x:v>
@@ -16438,7 +16441,7 @@
     </x:row>
     <x:row r="144" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A144" s="99" t="n">
-        <x:v>143</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B144" s="20" t="str">
         <x:v>Konata Mumpfield</x:v>
@@ -16526,7 +16529,7 @@
     </x:row>
     <x:row r="146" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A146" s="99" t="n">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B146" s="20" t="str">
         <x:v>Luke McCaffrey</x:v>
@@ -16570,7 +16573,7 @@
     </x:row>
     <x:row r="147" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A147" s="99" t="n">
-        <x:v>146</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B147" s="20" t="str">
         <x:v>Tom Kennedy</x:v>
@@ -16614,7 +16617,7 @@
     </x:row>
     <x:row r="148" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A148" s="99" t="n">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B148" s="20" t="str">
         <x:v>Jalen Royals</x:v>
@@ -16658,7 +16661,7 @@
     </x:row>
     <x:row r="149" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A149" s="99" t="n">
-        <x:v>148</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B149" s="20" t="str">
         <x:v>Deion Burks</x:v>
@@ -16702,7 +16705,7 @@
     </x:row>
     <x:row r="150" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A150" s="99" t="n">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B150" s="20" t="str">
         <x:v>Eric Rivers Jr.</x:v>
@@ -16790,7 +16793,7 @@
     </x:row>
     <x:row r="152" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A152" s="99" t="n">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B152" s="20" t="str">
         <x:v>Isaiah Bond</x:v>
@@ -16834,7 +16837,7 @@
     </x:row>
     <x:row r="153" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A153" s="99" t="n">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B153" s="20" t="str">
         <x:v>David Sills V</x:v>
@@ -16878,7 +16881,7 @@
     </x:row>
     <x:row r="154" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A154" s="99" t="n">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B154" s="20" t="str">
         <x:v>JP Richardson</x:v>
@@ -16922,7 +16925,7 @@
     </x:row>
     <x:row r="155" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A155" s="99" t="n">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B155" s="20" t="str">
         <x:v>Keandre Lambert-Smith</x:v>
@@ -16966,7 +16969,7 @@
     </x:row>
     <x:row r="156" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A156" s="99" t="n">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B156" s="20" t="str">
         <x:v>Marquez Valdes-Scantling</x:v>
@@ -17010,7 +17013,7 @@
     </x:row>
     <x:row r="157" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A157" s="99" t="n">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B157" s="20" t="str">
         <x:v>Xavier Weaver</x:v>
@@ -17054,7 +17057,7 @@
     </x:row>
     <x:row r="158" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A158" s="99" t="n">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B158" s="20" t="str">
         <x:v>Tez Johnson</x:v>
@@ -17098,7 +17101,7 @@
     </x:row>
     <x:row r="159" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A159" s="99" t="n">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B159" s="20" t="str">
         <x:v>Kevin Austin Jr.</x:v>
@@ -17142,7 +17145,7 @@
     </x:row>
     <x:row r="160" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A160" s="99" t="n">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B160" s="20" t="str">
         <x:v>Lil'Jordan Humphrey</x:v>
@@ -17230,7 +17233,7 @@
     </x:row>
     <x:row r="162" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A162" s="99" t="n">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B162" s="20" t="str">
         <x:v>Ben Skowronek</x:v>
@@ -17274,7 +17277,7 @@
     </x:row>
     <x:row r="163" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A163" s="99" t="n">
-        <x:v>162</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B163" s="20" t="str">
         <x:v>Greg Dortch</x:v>
@@ -17318,7 +17321,7 @@
     </x:row>
     <x:row r="164" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A164" s="99" t="n">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B164" s="20" t="str">
         <x:v>Zay Jones</x:v>
@@ -17362,7 +17365,7 @@
     </x:row>
     <x:row r="165" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A165" s="99" t="n">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B165" s="20" t="str">
         <x:v>Bo Melton</x:v>
@@ -17406,7 +17409,7 @@
     </x:row>
     <x:row r="166" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A166" s="99" t="n">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B166" s="20" t="str">
         <x:v>Colbie Young</x:v>
@@ -17450,7 +17453,7 @@
     </x:row>
     <x:row r="167" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A167" s="99" t="n">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B167" s="20" t="str">
         <x:v>Reggie Virgil</x:v>
@@ -17538,7 +17541,7 @@
     </x:row>
     <x:row r="169" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A169" s="99" t="n">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B169" s="20" t="str">
         <x:v>Elijah Moore</x:v>
@@ -17582,7 +17585,7 @@
     </x:row>
     <x:row r="170" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A170" s="99" t="n">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B170" s="20" t="str">
         <x:v>Sterling Shepard</x:v>
@@ -17626,7 +17629,7 @@
     </x:row>
     <x:row r="171" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A171" s="99" t="n">
-        <x:v>170</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B171" s="20" t="str">
         <x:v>Jimmy Horn Jr.</x:v>
@@ -17670,7 +17673,7 @@
     </x:row>
     <x:row r="172" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A172" s="99" t="n">
-        <x:v>171</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B172" s="20" t="str">
         <x:v>Noah Thomas</x:v>
@@ -17714,7 +17717,7 @@
     </x:row>
     <x:row r="173" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A173" s="99" t="n">
-        <x:v>172</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B173" s="20" t="str">
         <x:v>Tai Felton</x:v>
@@ -17758,7 +17761,7 @@
     </x:row>
     <x:row r="174" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A174" s="99" t="n">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B174" s="20" t="str">
         <x:v>CJ Daniels</x:v>
@@ -17802,7 +17805,7 @@
     </x:row>
     <x:row r="175" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A175" s="99" t="n">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B175" s="20" t="str">
         <x:v>Isaiah Williams</x:v>
@@ -17934,7 +17937,7 @@
     </x:row>
     <x:row r="178" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A178" s="99" t="n">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B178" s="20" t="str">
         <x:v>Tyrell Shavers</x:v>
@@ -17978,7 +17981,7 @@
     </x:row>
     <x:row r="179" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A179" s="99" t="n">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B179" s="20" t="str">
         <x:v>Cody White</x:v>
@@ -18022,7 +18025,7 @@
     </x:row>
     <x:row r="180" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A180" s="99" t="n">
-        <x:v>179</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B180" s="20" t="str">
         <x:v>Malachi Corley</x:v>
@@ -18110,7 +18113,7 @@
     </x:row>
     <x:row r="182" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A182" s="99" t="n">
-        <x:v>181</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B182" s="20" t="str">
         <x:v>Mason Tipton</x:v>
@@ -18154,7 +18157,7 @@
     </x:row>
     <x:row r="183" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A183" s="99" t="n">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B183" s="20" t="str">
         <x:v>David Moore</x:v>
@@ -18198,7 +18201,7 @@
     </x:row>
     <x:row r="184" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A184" s="99" t="n">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="B184" s="20" t="str">
         <x:v>Jonathan Mingo</x:v>
@@ -18242,7 +18245,7 @@
     </x:row>
     <x:row r="185" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A185" s="99" t="n">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B185" s="20" t="str">
         <x:v>Chase Roberts</x:v>
@@ -18286,7 +18289,7 @@
     </x:row>
     <x:row r="186" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A186" s="99" t="n">
-        <x:v>185</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B186" s="20" t="str">
         <x:v>Kaden Wetjen</x:v>
@@ -18330,7 +18333,7 @@
     </x:row>
     <x:row r="187" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A187" s="99" t="n">
-        <x:v>186</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B187" s="20" t="str">
         <x:v>Anthony Gould</x:v>
@@ -18418,7 +18421,7 @@
     </x:row>
     <x:row r="189" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A189" s="99" t="n">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="B189" s="20" t="str">
         <x:v>Tyler Johnson</x:v>
@@ -18462,7 +18465,7 @@
     </x:row>
     <x:row r="190" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A190" s="99" t="n">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B190" s="20" t="str">
         <x:v>Justin Watson</x:v>
@@ -18506,7 +18509,7 @@
     </x:row>
     <x:row r="191" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A191" s="99" t="n">
-        <x:v>190</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B191" s="20" t="str">
         <x:v>Jake Bobo</x:v>
@@ -18726,7 +18729,7 @@
     </x:row>
     <x:row r="196" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A196" s="99" t="n">
-        <x:v>195</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B196" s="20" t="str">
         <x:v>Arian Smith</x:v>
@@ -18770,7 +18773,7 @@
     </x:row>
     <x:row r="197" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A197" s="99" t="n">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B197" s="20" t="str">
         <x:v>Chris Moore</x:v>
@@ -18814,7 +18817,7 @@
     </x:row>
     <x:row r="198" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A198" s="99" t="n">
-        <x:v>197</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B198" s="20" t="str">
         <x:v>Ricky White III</x:v>
@@ -18902,7 +18905,7 @@
     </x:row>
     <x:row r="200" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A200" s="99" t="n">
-        <x:v>199</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B200" s="20" t="str">
         <x:v>Emmanuel Henderson Jr.</x:v>
@@ -18946,7 +18949,7 @@
     </x:row>
     <x:row r="201" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A201" s="99" t="n">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="B201" s="20" t="str">
         <x:v>Bryce Oliver</x:v>
@@ -18990,7 +18993,7 @@
     </x:row>
     <x:row r="202" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A202" s="99" t="n">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B202" s="20" t="str">
         <x:v>Jordan Watkins</x:v>
@@ -19034,7 +19037,7 @@
     </x:row>
     <x:row r="203" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A203" s="99" t="n">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B203" s="20" t="str">
         <x:v>Kameron Johnson</x:v>
@@ -19078,7 +19081,7 @@
     </x:row>
     <x:row r="204" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A204" s="99" t="n">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B204" s="20" t="str">
         <x:v>JuJu Smith-Schuster</x:v>
@@ -19122,7 +19125,7 @@
     </x:row>
     <x:row r="205" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A205" s="99" t="n">
-        <x:v>204</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B205" s="20" t="str">
         <x:v>Jayden Higgins</x:v>
@@ -19166,7 +19169,7 @@
     </x:row>
     <x:row r="206" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A206" s="99" t="n">
-        <x:v>205</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B206" s="20" t="str">
         <x:v>A.T. Perry</x:v>
@@ -19210,7 +19213,7 @@
     </x:row>
     <x:row r="207" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A207" s="99" t="n">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B207" s="20" t="str">
         <x:v>Anthony Smith</x:v>
@@ -19254,7 +19257,7 @@
     </x:row>
     <x:row r="208" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A208" s="99" t="n">
-        <x:v>207</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B208" s="20" t="str">
         <x:v>Braxton Berrios</x:v>
@@ -19298,7 +19301,7 @@
     </x:row>
     <x:row r="209" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A209" s="99" t="n">
-        <x:v>208</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="B209" s="20" t="str">
         <x:v>Britain Covey</x:v>
@@ -19342,7 +19345,7 @@
     </x:row>
     <x:row r="210" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A210" s="99" t="n">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B210" s="20" t="str">
         <x:v>Casey Washington</x:v>
@@ -19386,7 +19389,7 @@
     </x:row>
     <x:row r="211" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A211" s="99" t="n">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B211" s="20" t="str">
         <x:v>Cedrick Wilson Jr.</x:v>
@@ -19430,7 +19433,7 @@
     </x:row>
     <x:row r="212" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A212" s="99" t="n">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B212" s="20" t="str">
         <x:v>Charlie Jones</x:v>
@@ -19474,7 +19477,7 @@
     </x:row>
     <x:row r="213" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A213" s="99" t="n">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="B213" s="20" t="str">
         <x:v>Chris Brazzell II</x:v>
@@ -19518,7 +19521,7 @@
     </x:row>
     <x:row r="214" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A214" s="99" t="n">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="B214" s="20" t="str">
         <x:v>Danny Gray</x:v>
@@ -19562,7 +19565,7 @@
     </x:row>
     <x:row r="215" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A215" s="99" t="n">
-        <x:v>214</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B215" s="20" t="str">
         <x:v>Dante Pettis</x:v>
@@ -19606,7 +19609,7 @@
     </x:row>
     <x:row r="216" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A216" s="99" t="n">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B216" s="20" t="str">
         <x:v>Dareke Young</x:v>
@@ -19650,7 +19653,7 @@
     </x:row>
     <x:row r="217" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A217" s="99" t="n">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="B217" s="20" t="str">
         <x:v>Deven Thompkins</x:v>
@@ -19694,7 +19697,7 @@
     </x:row>
     <x:row r="218" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A218" s="99" t="n">
-        <x:v>217</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B218" s="20" t="str">
         <x:v>Devin Duvernay</x:v>
@@ -19738,7 +19741,7 @@
     </x:row>
     <x:row r="219" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A219" s="99" t="n">
-        <x:v>218</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B219" s="20" t="str">
         <x:v>Dominic Lovett</x:v>
@@ -19782,7 +19785,7 @@
     </x:row>
     <x:row r="220" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A220" s="99" t="n">
-        <x:v>219</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="B220" s="20" t="str">
         <x:v>Efton Chism III</x:v>
@@ -19826,7 +19829,7 @@
     </x:row>
     <x:row r="221" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A221" s="99" t="n">
-        <x:v>220</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B221" s="20" t="str">
         <x:v>Gage Larvadain</x:v>
@@ -19870,7 +19873,7 @@
     </x:row>
     <x:row r="222" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A222" s="99" t="n">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B222" s="20" t="str">
         <x:v>Gunner Olszewski</x:v>
@@ -19914,7 +19917,7 @@
     </x:row>
     <x:row r="223" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A223" s="99" t="n">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B223" s="20" t="str">
         <x:v>Ihmir Smith-Marsette</x:v>
@@ -19958,7 +19961,7 @@
     </x:row>
     <x:row r="224" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A224" s="99" t="n">
-        <x:v>223</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B224" s="20" t="str">
         <x:v>Irv Charles</x:v>
@@ -20002,7 +20005,7 @@
     </x:row>
     <x:row r="225" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A225" s="99" t="n">
-        <x:v>224</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B225" s="20" t="str">
         <x:v>Isaiah Neyor</x:v>
@@ -20046,7 +20049,7 @@
     </x:row>
     <x:row r="226" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A226" s="99" t="n">
-        <x:v>225</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="B226" s="20" t="str">
         <x:v>Jacob Cowing</x:v>
@@ -20090,7 +20093,7 @@
     </x:row>
     <x:row r="227" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A227" s="99" t="n">
-        <x:v>226</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B227" s="20" t="str">
         <x:v>Jalen Brooks</x:v>
@@ -20134,7 +20137,7 @@
     </x:row>
     <x:row r="228" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A228" s="99" t="n">
-        <x:v>227</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="B228" s="20" t="str">
         <x:v>Jalin Hyatt</x:v>
@@ -20178,7 +20181,7 @@
     </x:row>
     <x:row r="229" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A229" s="99" t="n">
-        <x:v>228</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="B229" s="20" t="str">
         <x:v>Jamari Thrash</x:v>
@@ -20222,7 +20225,7 @@
     </x:row>
     <x:row r="230" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A230" s="99" t="n">
-        <x:v>229</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B230" s="20" t="str">
         <x:v>Jason Brownlee</x:v>
@@ -21411,7 +21414,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0c708d7afd24196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6636e7ee4f8e42ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28331,7 +28334,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bd1d8da4af4175"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1e10696af80409d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28375,7 +28378,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B2" s="46" t="str">
-        <x:v>August 24, 2026, 10:46 AM ET</x:v>
+        <x:v>August 30, 2026, 12:00 PM ET</x:v>
       </x:c>
       <x:c r="C2" s="46" t="str">
         <x:v>Timezone</x:v>
@@ -32886,6 +32889,120 @@
       <x:c r="K132"/>
       <x:c r="L132"/>
     </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>Kayshon Boutte</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>HOU</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>TEAM UPDATED</x:v>
+      </x:c>
+      <x:c r="E133" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="F133" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="G133" t="n">
+        <x:v>73.9</x:v>
+      </x:c>
+      <x:c r="H133" t="n">
+        <x:v>73.9</x:v>
+      </x:c>
+      <x:c r="I133" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J133" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K133" t="str">
+        <x:v>Team updated after Houston officially acquired Boutte from New England; workload projection is unchanged pending role evidence.</x:v>
+      </x:c>
+      <x:c r="L133" t="str">
+        <x:v>https://www.houstontexans.com/news/houston-texans-transactions-8-25-2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>Tutu Atwell</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>LAR</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>TEAM UPDATED</x:v>
+      </x:c>
+      <x:c r="E134" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F134" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="G134" t="n">
+        <x:v>33.9</x:v>
+      </x:c>
+      <x:c r="H134" t="n">
+        <x:v>33.9</x:v>
+      </x:c>
+      <x:c r="I134" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J134" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K134" t="str">
+        <x:v>Team updated after the Rams officially reacquired Atwell from Miami; workload projection is unchanged pending role evidence.</x:v>
+      </x:c>
+      <x:c r="L134" t="str">
+        <x:v>https://www.therams.com/news/rams-agree-to-trade-rb-jarquez-hunter-to-dolphins-for-wr-tutu-atwell</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>Cedric Tillman</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>FA</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>REMOVED FROM ACTIVE PROJECTION</x:v>
+      </x:c>
+      <x:c r="E135" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F135" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="G135" t="n">
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="H135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I135" t="n">
+        <x:v>-68.8</x:v>
+      </x:c>
+      <x:c r="J135" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K135" t="str">
+        <x:v>Cleveland waived Tillman, so his active-team workload is removed until he signs elsewhere and a new role is established.</x:v>
+      </x:c>
+      <x:c r="L135" t="str">
+        <x:v>https://x.com/DanielOyefusi/status/2093081141716660460</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A54:L54"/>

</xml_diff>

<commit_message>
Refresh NFL projections rankings and ADP (#108)
Co-authored-by: Codex <codex@openai.com>
</commit_message>
<xml_diff>
--- a/data/projections.xlsx
+++ b/data/projections.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QB" sheetId="1" r:id="R2a696b901a2c40b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="2" r:id="Rd38ac66a6b174ff8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WR" sheetId="3" r:id="Rc46ecbfbe24f493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TE" sheetId="4" r:id="R9835e52518b8415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Update" sheetId="5" r:id="R24a4ed4641cb4d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QB" sheetId="1" r:id="R7d43bf37c6254be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RB" sheetId="2" r:id="Rdf682e3a2cba453a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WR" sheetId="3" r:id="R7593fea4eea94747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TE" sheetId="4" r:id="R9ca4e15c1c1646d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Update" sheetId="5" r:id="R6281eb41920041b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2599,7 +2599,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1488efdaa88246e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44035cbc9ecb426f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10091,7 +10091,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bf03de1462243f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf335419fd37e4d05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10366,7 +10366,7 @@
     </x:row>
     <x:row r="6" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A6" s="99" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B6" s="20" t="str">
         <x:v>Justin Jefferson</x:v>
@@ -10410,7 +10410,7 @@
     </x:row>
     <x:row r="7" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A7" s="99" t="n">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="20" t="str">
         <x:v>Nico Collins</x:v>
@@ -10586,7 +10586,7 @@
     </x:row>
     <x:row r="11" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A11" s="99" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B11" s="20" t="str">
         <x:v>Chris Olave</x:v>
@@ -10630,7 +10630,7 @@
     </x:row>
     <x:row r="12" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A12" s="99" t="n">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B12" s="20" t="str">
         <x:v>A.J. Brown</x:v>
@@ -10806,7 +10806,7 @@
     </x:row>
     <x:row r="16" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A16" s="99" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B16" s="20" t="str">
         <x:v>DeVonta Smith</x:v>
@@ -10850,7 +10850,7 @@
     </x:row>
     <x:row r="17" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A17" s="99" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B17" s="20" t="str">
         <x:v>Garrett Wilson</x:v>
@@ -10894,7 +10894,7 @@
     </x:row>
     <x:row r="18" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A18" s="99" t="n">
-        <x:v>17</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B18" s="20" t="str">
         <x:v>Tee Higgins</x:v>
@@ -10938,7 +10938,7 @@
     </x:row>
     <x:row r="19" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A19" s="99" t="n">
-        <x:v>18</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B19" s="20" t="str">
         <x:v>Marvin Harrison Jr.</x:v>
@@ -11070,7 +11070,7 @@
     </x:row>
     <x:row r="22" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A22" s="99" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B22" s="20" t="str">
         <x:v>Luther Burden III</x:v>
@@ -11114,7 +11114,7 @@
     </x:row>
     <x:row r="23" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A23" s="99" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B23" s="20" t="str">
         <x:v>DJ Moore</x:v>
@@ -11158,7 +11158,7 @@
     </x:row>
     <x:row r="24" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A24" s="99" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B24" s="20" t="str">
         <x:v>Terry McLaurin</x:v>
@@ -11202,7 +11202,7 @@
     </x:row>
     <x:row r="25" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A25" s="99" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B25" s="20" t="str">
         <x:v>Malik Nabers</x:v>
@@ -11246,7 +11246,7 @@
     </x:row>
     <x:row r="26" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A26" s="99" t="n">
-        <x:v>25</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B26" s="20" t="str">
         <x:v>Jameson Williams</x:v>
@@ -11334,7 +11334,7 @@
     </x:row>
     <x:row r="28" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A28" s="99" t="n">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B28" s="20" t="str">
         <x:v>Ladd McConkey</x:v>
@@ -11378,7 +11378,7 @@
     </x:row>
     <x:row r="29" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A29" s="99" t="n">
-        <x:v>28</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B29" s="20" t="str">
         <x:v>Mike Evans</x:v>
@@ -11422,7 +11422,7 @@
     </x:row>
     <x:row r="30" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A30" s="99" t="n">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B30" s="20" t="str">
         <x:v>Courtland Sutton</x:v>
@@ -11466,7 +11466,7 @@
     </x:row>
     <x:row r="31" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A31" s="99" t="n">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B31" s="20" t="str">
         <x:v>Wan'Dale Robinson</x:v>
@@ -11510,7 +11510,7 @@
     </x:row>
     <x:row r="32" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A32" s="99" t="n">
-        <x:v>31</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B32" s="20" t="str">
         <x:v>Davante Adams</x:v>
@@ -11554,7 +11554,7 @@
     </x:row>
     <x:row r="33" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A33" s="99" t="n">
-        <x:v>32</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B33" s="20" t="str">
         <x:v>DK Metcalf</x:v>
@@ -11598,7 +11598,7 @@
     </x:row>
     <x:row r="34" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A34" s="99" t="n">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B34" s="20" t="str">
         <x:v>Christian Watson</x:v>
@@ -11642,7 +11642,7 @@
     </x:row>
     <x:row r="35" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A35" s="99" t="n">
-        <x:v>34</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B35" s="20" t="str">
         <x:v>Michael Wilson</x:v>
@@ -11686,7 +11686,7 @@
     </x:row>
     <x:row r="36" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A36" s="99" t="n">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B36" s="20" t="str">
         <x:v>Michael Pittman Jr.</x:v>
@@ -11730,7 +11730,7 @@
     </x:row>
     <x:row r="37" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A37" s="99" t="n">
-        <x:v>36</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B37" s="20" t="str">
         <x:v>Parker Washington</x:v>
@@ -11774,7 +11774,7 @@
     </x:row>
     <x:row r="38" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A38" s="99" t="n">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B38" s="20" t="str">
         <x:v>Brian Thomas Jr.</x:v>
@@ -11862,7 +11862,7 @@
     </x:row>
     <x:row r="40" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A40" s="99" t="n">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B40" s="20" t="str">
         <x:v>Matthew Golden</x:v>
@@ -11906,7 +11906,7 @@
     </x:row>
     <x:row r="41" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A41" s="99" t="n">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B41" s="20" t="str">
         <x:v>Jordan Addison</x:v>
@@ -11950,7 +11950,7 @@
     </x:row>
     <x:row r="42" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A42" s="99" t="n">
-        <x:v>41</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B42" s="20" t="str">
         <x:v>Alec Pierce</x:v>
@@ -12038,7 +12038,7 @@
     </x:row>
     <x:row r="44" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A44" s="99" t="n">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B44" s="20" t="str">
         <x:v>Josh Downs</x:v>
@@ -12082,7 +12082,7 @@
     </x:row>
     <x:row r="45" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A45" s="99" t="n">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B45" s="20" t="str">
         <x:v>Stefon Diggs</x:v>
@@ -12126,7 +12126,7 @@
     </x:row>
     <x:row r="46" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A46" s="99" t="n">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B46" s="20" t="str">
         <x:v>Tre Tucker</x:v>
@@ -12170,7 +12170,7 @@
     </x:row>
     <x:row r="47" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A47" s="99" t="n">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B47" s="20" t="str">
         <x:v>Xavier Worthy</x:v>
@@ -12258,7 +12258,7 @@
     </x:row>
     <x:row r="49" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A49" s="99" t="n">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B49" s="20" t="str">
         <x:v>Chris Godwin Jr.</x:v>
@@ -12302,7 +12302,7 @@
     </x:row>
     <x:row r="50" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A50" s="99" t="n">
-        <x:v>49</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B50" s="20" t="str">
         <x:v>Adonai Mitchell</x:v>
@@ -12346,7 +12346,7 @@
     </x:row>
     <x:row r="51" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A51" s="99" t="n">
-        <x:v>50</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B51" s="20" t="str">
         <x:v>Carnell Tate</x:v>
@@ -12390,7 +12390,7 @@
     </x:row>
     <x:row r="52" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A52" s="99" t="n">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B52" s="20" t="str">
         <x:v>Khalil Shakir</x:v>
@@ -12478,7 +12478,7 @@
     </x:row>
     <x:row r="54" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A54" s="99" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B54" s="20" t="str">
         <x:v>Denzel Boston</x:v>
@@ -12522,7 +12522,7 @@
     </x:row>
     <x:row r="55" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A55" s="99" t="n">
-        <x:v>54</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B55" s="20" t="str">
         <x:v>Rashid Shaheed</x:v>
@@ -12654,7 +12654,7 @@
     </x:row>
     <x:row r="58" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A58" s="99" t="n">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B58" s="20" t="str">
         <x:v>Keenan Allen</x:v>
@@ -12698,7 +12698,7 @@
     </x:row>
     <x:row r="59" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A59" s="99" t="n">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B59" s="20" t="str">
         <x:v>Tank Dell</x:v>
@@ -12742,7 +12742,7 @@
     </x:row>
     <x:row r="60" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A60" s="99" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B60" s="20" t="str">
         <x:v>KC Concepcion</x:v>
@@ -12786,7 +12786,7 @@
     </x:row>
     <x:row r="61" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A61" s="99" t="n">
-        <x:v>60</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B61" s="20" t="str">
         <x:v>Calvin Ridley</x:v>
@@ -12918,7 +12918,7 @@
     </x:row>
     <x:row r="64" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A64" s="99" t="n">
-        <x:v>63</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B64" s="20" t="str">
         <x:v>John Metchie III</x:v>
@@ -12962,7 +12962,7 @@
     </x:row>
     <x:row r="65" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A65" s="99" t="n">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B65" s="20" t="str">
         <x:v>Zachariah Branch</x:v>
@@ -13006,7 +13006,7 @@
     </x:row>
     <x:row r="66" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A66" s="99" t="n">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B66" s="20" t="str">
         <x:v>Deebo Samuel Sr.</x:v>
@@ -13050,7 +13050,7 @@
     </x:row>
     <x:row r="67" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A67" s="99" t="n">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B67" s="20" t="str">
         <x:v>Jalen Coker</x:v>
@@ -13094,7 +13094,7 @@
     </x:row>
     <x:row r="68" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A68" s="99" t="n">
-        <x:v>67</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B68" s="20" t="str">
         <x:v>Romeo Doubs</x:v>
@@ -13138,7 +13138,7 @@
     </x:row>
     <x:row r="69" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A69" s="99" t="n">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B69" s="20" t="str">
         <x:v>Omar Cooper Jr.</x:v>
@@ -13182,7 +13182,7 @@
     </x:row>
     <x:row r="70" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A70" s="99" t="n">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B70" s="20" t="str">
         <x:v>Jalen McMillan</x:v>
@@ -13226,7 +13226,7 @@
     </x:row>
     <x:row r="71" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A71" s="99" t="n">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B71" s="20" t="str">
         <x:v>Andrei Iosivas</x:v>
@@ -13270,7 +13270,7 @@
     </x:row>
     <x:row r="72" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A72" s="99" t="n">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B72" s="20" t="str">
         <x:v>Rashod Bateman</x:v>
@@ -13314,7 +13314,7 @@
     </x:row>
     <x:row r="73" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A73" s="99" t="n">
-        <x:v>72</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B73" s="20" t="str">
         <x:v>Malik Washington</x:v>
@@ -13358,7 +13358,7 @@
     </x:row>
     <x:row r="74" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A74" s="99" t="n">
-        <x:v>73</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B74" s="20" t="str">
         <x:v>Ted Hurst</x:v>
@@ -13402,7 +13402,7 @@
     </x:row>
     <x:row r="75" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A75" s="99" t="n">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B75" s="20" t="str">
         <x:v>Theo Wease Jr.</x:v>
@@ -13490,7 +13490,7 @@
     </x:row>
     <x:row r="77" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A77" s="99" t="n">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B77" s="20" t="str">
         <x:v>Troy Franklin</x:v>
@@ -13534,7 +13534,7 @@
     </x:row>
     <x:row r="78" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A78" s="99" t="n">
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B78" s="20" t="str">
         <x:v>Malik Benson</x:v>
@@ -13578,7 +13578,7 @@
     </x:row>
     <x:row r="79" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A79" s="99" t="n">
-        <x:v>78</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B79" s="20" t="str">
         <x:v>Christian Kirk</x:v>
@@ -13622,7 +13622,7 @@
     </x:row>
     <x:row r="80" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A80" s="99" t="n">
-        <x:v>79</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B80" s="20" t="str">
         <x:v>Isaac TeSlaa</x:v>
@@ -13666,7 +13666,7 @@
     </x:row>
     <x:row r="81" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A81" s="99" t="n">
-        <x:v>80</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B81" s="20" t="str">
         <x:v>Ja'Kobi Lane</x:v>
@@ -13710,7 +13710,7 @@
     </x:row>
     <x:row r="82" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A82" s="99" t="n">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B82" s="20" t="str">
         <x:v>Jaylin Noel</x:v>
@@ -13754,7 +13754,7 @@
     </x:row>
     <x:row r="83" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A83" s="99" t="n">
-        <x:v>82</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B83" s="20" t="str">
         <x:v>Dontayvion Wicks</x:v>
@@ -13798,7 +13798,7 @@
     </x:row>
     <x:row r="84" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A84" s="99" t="n">
-        <x:v>83</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B84" s="20" t="str">
         <x:v>Jack Bech</x:v>
@@ -13842,7 +13842,7 @@
     </x:row>
     <x:row r="85" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A85" s="99" t="n">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B85" s="20" t="str">
         <x:v>Cooper Kupp</x:v>
@@ -13886,7 +13886,7 @@
     </x:row>
     <x:row r="86" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A86" s="99" t="n">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B86" s="20" t="str">
         <x:v>De'Zhaun Stribling</x:v>
@@ -13930,7 +13930,7 @@
     </x:row>
     <x:row r="87" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A87" s="99" t="n">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B87" s="20" t="str">
         <x:v>Jordyn Tyson</x:v>
@@ -13974,13 +13974,13 @@
     </x:row>
     <x:row r="88" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A88" s="99" t="n">
-        <x:v>87</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B88" s="20" t="str">
         <x:v>Kayshon Boutte</x:v>
       </x:c>
       <x:c r="C88" s="16" t="str">
-        <x:v>NE</x:v>
+        <x:v>HOU</x:v>
       </x:c>
       <x:c r="D88" s="100" t="n">
         <x:v>33.7</x:v>
@@ -14018,7 +14018,7 @@
     </x:row>
     <x:row r="89" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A89" s="99" t="n">
-        <x:v>88</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B89" s="20" t="str">
         <x:v>Tyquan Thornton</x:v>
@@ -14106,7 +14106,7 @@
     </x:row>
     <x:row r="91" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A91" s="99" t="n">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B91" s="20" t="str">
         <x:v>Caleb Douglas</x:v>
@@ -14194,7 +14194,7 @@
     </x:row>
     <x:row r="93" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A93" s="99" t="n">
-        <x:v>92</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B93" s="20" t="str">
         <x:v>Elic Ayomanor</x:v>
@@ -14238,25 +14238,25 @@
     </x:row>
     <x:row r="94" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A94" s="99" t="n">
-        <x:v>93</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="B94" s="20" t="str">
         <x:v>Cedric Tillman</x:v>
       </x:c>
       <x:c r="C94" s="16" t="str">
-        <x:v>CLE</x:v>
+        <x:v>FA</x:v>
       </x:c>
       <x:c r="D94" s="100" t="n">
-        <x:v>43.2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E94" s="100" t="n">
-        <x:v>24.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F94" s="100" t="n">
-        <x:v>301.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G94" s="100" t="n">
-        <x:v>2.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H94" s="100" t="n">
         <x:v>0</x:v>
@@ -14271,18 +14271,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L94" s="100" t="n">
-        <x:v>68.8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M94" s="100" t="n">
-        <x:v>56.4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N94" s="101" t="n">
-        <x:v>43.9</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O94" t="n">
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="95" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A95" s="99" t="n">
-        <x:v>94</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B95" s="20" t="str">
         <x:v>Hollywood Brown</x:v>
@@ -14326,7 +14329,7 @@
     </x:row>
     <x:row r="96" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A96" s="99" t="n">
-        <x:v>95</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B96" s="20" t="str">
         <x:v>Mack Hollins</x:v>
@@ -14370,7 +14373,7 @@
     </x:row>
     <x:row r="97" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A97" s="99" t="n">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B97" s="20" t="str">
         <x:v>Travis Hunter</x:v>
@@ -14414,7 +14417,7 @@
     </x:row>
     <x:row r="98" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A98" s="99" t="n">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B98" s="20" t="str">
         <x:v>Joshua Palmer</x:v>
@@ -14458,7 +14461,7 @@
     </x:row>
     <x:row r="99" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A99" s="99" t="n">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B99" s="20" t="str">
         <x:v>Jalen Tolbert</x:v>
@@ -14502,7 +14505,7 @@
     </x:row>
     <x:row r="100" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A100" s="99" t="n">
-        <x:v>99</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B100" s="20" t="str">
         <x:v>Xavier Hutchinson</x:v>
@@ -14546,7 +14549,7 @@
     </x:row>
     <x:row r="101" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A101" s="99" t="n">
-        <x:v>100</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B101" s="20" t="str">
         <x:v>Chimere Dike</x:v>
@@ -14634,7 +14637,7 @@
     </x:row>
     <x:row r="103" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A103" s="99" t="n">
-        <x:v>102</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B103" s="20" t="str">
         <x:v>Xavier Legette</x:v>
@@ -14678,7 +14681,7 @@
     </x:row>
     <x:row r="104" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A104" s="99" t="n">
-        <x:v>103</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B104" s="20" t="str">
         <x:v>Pat Bryant</x:v>
@@ -14766,7 +14769,7 @@
     </x:row>
     <x:row r="106" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A106" s="99" t="n">
-        <x:v>105</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B106" s="20" t="str">
         <x:v>Jahdae Walker</x:v>
@@ -14810,7 +14813,7 @@
     </x:row>
     <x:row r="107" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A107" s="99" t="n">
-        <x:v>106</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B107" s="20" t="str">
         <x:v>Elijah Sarratt</x:v>
@@ -14854,7 +14857,7 @@
     </x:row>
     <x:row r="108" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A108" s="99" t="n">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B108" s="20" t="str">
         <x:v>Keon Coleman</x:v>
@@ -14898,7 +14901,7 @@
     </x:row>
     <x:row r="109" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A109" s="99" t="n">
-        <x:v>108</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B109" s="20" t="str">
         <x:v>Kendrick Bourne</x:v>
@@ -14942,7 +14945,7 @@
     </x:row>
     <x:row r="110" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A110" s="99" t="n">
-        <x:v>109</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B110" s="20" t="str">
         <x:v>Jahan Dotson</x:v>
@@ -14986,7 +14989,7 @@
     </x:row>
     <x:row r="111" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A111" s="99" t="n">
-        <x:v>110</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B111" s="20" t="str">
         <x:v>Olamide Zaccheaus</x:v>
@@ -15030,7 +15033,7 @@
     </x:row>
     <x:row r="112" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A112" s="99" t="n">
-        <x:v>111</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B112" s="20" t="str">
         <x:v>Savion Williams</x:v>
@@ -15074,7 +15077,7 @@
     </x:row>
     <x:row r="113" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A113" s="99" t="n">
-        <x:v>112</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B113" s="20" t="str">
         <x:v>Darnell Mooney</x:v>
@@ -15118,7 +15121,7 @@
     </x:row>
     <x:row r="114" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A114" s="99" t="n">
-        <x:v>113</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B114" s="20" t="str">
         <x:v>Devaughn Vele</x:v>
@@ -15162,7 +15165,7 @@
     </x:row>
     <x:row r="115" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A115" s="99" t="n">
-        <x:v>114</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B115" s="20" t="str">
         <x:v>Malachi Fields</x:v>
@@ -15206,7 +15209,7 @@
     </x:row>
     <x:row r="116" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A116" s="99" t="n">
-        <x:v>115</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B116" s="20" t="str">
         <x:v>Tory Horton</x:v>
@@ -15250,7 +15253,7 @@
     </x:row>
     <x:row r="117" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A117" s="99" t="n">
-        <x:v>116</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B117" s="20" t="str">
         <x:v>Marvin Mims Jr.</x:v>
@@ -15294,7 +15297,7 @@
     </x:row>
     <x:row r="118" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A118" s="99" t="n">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B118" s="20" t="str">
         <x:v>Bub Means</x:v>
@@ -15382,7 +15385,7 @@
     </x:row>
     <x:row r="120" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A120" s="99" t="n">
-        <x:v>119</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B120" s="20" t="str">
         <x:v>Cyrus Allen</x:v>
@@ -15426,7 +15429,7 @@
     </x:row>
     <x:row r="121" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A121" s="99" t="n">
-        <x:v>120</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B121" s="20" t="str">
         <x:v>Kyle Williams</x:v>
@@ -15470,7 +15473,7 @@
     </x:row>
     <x:row r="122" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A122" s="99" t="n">
-        <x:v>121</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B122" s="20" t="str">
         <x:v>DeMario Douglas</x:v>
@@ -15602,7 +15605,7 @@
     </x:row>
     <x:row r="125" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A125" s="99" t="n">
-        <x:v>124</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B125" s="20" t="str">
         <x:v>KaVontae Turpin</x:v>
@@ -15646,7 +15649,7 @@
     </x:row>
     <x:row r="126" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A126" s="99" t="n">
-        <x:v>125</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B126" s="20" t="str">
         <x:v>Calvin Austin III</x:v>
@@ -15822,7 +15825,7 @@
     </x:row>
     <x:row r="130" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A130" s="99" t="n">
-        <x:v>129</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B130" s="20" t="str">
         <x:v>Ashton Dulin</x:v>
@@ -15910,7 +15913,7 @@
     </x:row>
     <x:row r="132" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A132" s="99" t="n">
-        <x:v>131</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B132" s="20" t="str">
         <x:v>Dyami Brown</x:v>
@@ -15954,13 +15957,13 @@
     </x:row>
     <x:row r="133" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A133" s="99" t="n">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B133" s="20" t="str">
         <x:v>Tutu Atwell</x:v>
       </x:c>
       <x:c r="C133" s="16" t="str">
-        <x:v>MIA</x:v>
+        <x:v>LAR</x:v>
       </x:c>
       <x:c r="D133" s="100" t="n">
         <x:v>21.2</x:v>
@@ -15998,7 +16001,7 @@
     </x:row>
     <x:row r="134" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A134" s="99" t="n">
-        <x:v>133</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B134" s="20" t="str">
         <x:v>Odell Beckham Jr.</x:v>
@@ -16042,7 +16045,7 @@
     </x:row>
     <x:row r="135" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A135" s="99" t="n">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B135" s="20" t="str">
         <x:v>Kevin Coleman Jr.</x:v>
@@ -16086,7 +16089,7 @@
     </x:row>
     <x:row r="136" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A136" s="99" t="n">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B136" s="20" t="str">
         <x:v>Demarcus Robinson</x:v>
@@ -16130,7 +16133,7 @@
     </x:row>
     <x:row r="137" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A137" s="99" t="n">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B137" s="20" t="str">
         <x:v>Van Jefferson</x:v>
@@ -16174,7 +16177,7 @@
     </x:row>
     <x:row r="138" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A138" s="99" t="n">
-        <x:v>137</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B138" s="20" t="str">
         <x:v>Nick Westbrook-Ikhine</x:v>
@@ -16218,7 +16221,7 @@
     </x:row>
     <x:row r="139" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A139" s="99" t="n">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B139" s="20" t="str">
         <x:v>Treylon Burks</x:v>
@@ -16262,7 +16265,7 @@
     </x:row>
     <x:row r="140" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A140" s="99" t="n">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B140" s="20" t="str">
         <x:v>Zavion Thomas</x:v>
@@ -16306,7 +16309,7 @@
     </x:row>
     <x:row r="141" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A141" s="99" t="n">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B141" s="20" t="str">
         <x:v>Jaylin Lane</x:v>
@@ -16350,7 +16353,7 @@
     </x:row>
     <x:row r="142" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A142" s="99" t="n">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B142" s="20" t="str">
         <x:v>Dont'e Thornton Jr.</x:v>
@@ -16394,7 +16397,7 @@
     </x:row>
     <x:row r="143" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A143" s="99" t="n">
-        <x:v>142</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B143" s="20" t="str">
         <x:v>Tim Patrick</x:v>
@@ -16438,7 +16441,7 @@
     </x:row>
     <x:row r="144" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A144" s="99" t="n">
-        <x:v>143</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B144" s="20" t="str">
         <x:v>Konata Mumpfield</x:v>
@@ -16526,7 +16529,7 @@
     </x:row>
     <x:row r="146" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A146" s="99" t="n">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B146" s="20" t="str">
         <x:v>Luke McCaffrey</x:v>
@@ -16570,7 +16573,7 @@
     </x:row>
     <x:row r="147" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A147" s="99" t="n">
-        <x:v>146</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B147" s="20" t="str">
         <x:v>Tom Kennedy</x:v>
@@ -16614,7 +16617,7 @@
     </x:row>
     <x:row r="148" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A148" s="99" t="n">
-        <x:v>147</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B148" s="20" t="str">
         <x:v>Jalen Royals</x:v>
@@ -16658,7 +16661,7 @@
     </x:row>
     <x:row r="149" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A149" s="99" t="n">
-        <x:v>148</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B149" s="20" t="str">
         <x:v>Deion Burks</x:v>
@@ -16702,7 +16705,7 @@
     </x:row>
     <x:row r="150" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A150" s="99" t="n">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B150" s="20" t="str">
         <x:v>Eric Rivers Jr.</x:v>
@@ -16790,7 +16793,7 @@
     </x:row>
     <x:row r="152" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A152" s="99" t="n">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B152" s="20" t="str">
         <x:v>Isaiah Bond</x:v>
@@ -16834,7 +16837,7 @@
     </x:row>
     <x:row r="153" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A153" s="99" t="n">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B153" s="20" t="str">
         <x:v>David Sills V</x:v>
@@ -16878,7 +16881,7 @@
     </x:row>
     <x:row r="154" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A154" s="99" t="n">
-        <x:v>153</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B154" s="20" t="str">
         <x:v>JP Richardson</x:v>
@@ -16922,7 +16925,7 @@
     </x:row>
     <x:row r="155" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A155" s="99" t="n">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B155" s="20" t="str">
         <x:v>Keandre Lambert-Smith</x:v>
@@ -16966,7 +16969,7 @@
     </x:row>
     <x:row r="156" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A156" s="99" t="n">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B156" s="20" t="str">
         <x:v>Marquez Valdes-Scantling</x:v>
@@ -17010,7 +17013,7 @@
     </x:row>
     <x:row r="157" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A157" s="99" t="n">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B157" s="20" t="str">
         <x:v>Xavier Weaver</x:v>
@@ -17054,7 +17057,7 @@
     </x:row>
     <x:row r="158" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A158" s="99" t="n">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B158" s="20" t="str">
         <x:v>Tez Johnson</x:v>
@@ -17098,7 +17101,7 @@
     </x:row>
     <x:row r="159" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A159" s="99" t="n">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B159" s="20" t="str">
         <x:v>Kevin Austin Jr.</x:v>
@@ -17142,7 +17145,7 @@
     </x:row>
     <x:row r="160" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A160" s="99" t="n">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B160" s="20" t="str">
         <x:v>Lil'Jordan Humphrey</x:v>
@@ -17230,7 +17233,7 @@
     </x:row>
     <x:row r="162" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A162" s="99" t="n">
-        <x:v>161</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B162" s="20" t="str">
         <x:v>Ben Skowronek</x:v>
@@ -17274,7 +17277,7 @@
     </x:row>
     <x:row r="163" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A163" s="99" t="n">
-        <x:v>162</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B163" s="20" t="str">
         <x:v>Greg Dortch</x:v>
@@ -17318,7 +17321,7 @@
     </x:row>
     <x:row r="164" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A164" s="99" t="n">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B164" s="20" t="str">
         <x:v>Zay Jones</x:v>
@@ -17362,7 +17365,7 @@
     </x:row>
     <x:row r="165" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A165" s="99" t="n">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B165" s="20" t="str">
         <x:v>Bo Melton</x:v>
@@ -17406,7 +17409,7 @@
     </x:row>
     <x:row r="166" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A166" s="99" t="n">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B166" s="20" t="str">
         <x:v>Colbie Young</x:v>
@@ -17450,7 +17453,7 @@
     </x:row>
     <x:row r="167" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A167" s="99" t="n">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B167" s="20" t="str">
         <x:v>Reggie Virgil</x:v>
@@ -17538,7 +17541,7 @@
     </x:row>
     <x:row r="169" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A169" s="99" t="n">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B169" s="20" t="str">
         <x:v>Elijah Moore</x:v>
@@ -17582,7 +17585,7 @@
     </x:row>
     <x:row r="170" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A170" s="99" t="n">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B170" s="20" t="str">
         <x:v>Sterling Shepard</x:v>
@@ -17626,7 +17629,7 @@
     </x:row>
     <x:row r="171" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A171" s="99" t="n">
-        <x:v>170</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B171" s="20" t="str">
         <x:v>Jimmy Horn Jr.</x:v>
@@ -17670,7 +17673,7 @@
     </x:row>
     <x:row r="172" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A172" s="99" t="n">
-        <x:v>171</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B172" s="20" t="str">
         <x:v>Noah Thomas</x:v>
@@ -17714,7 +17717,7 @@
     </x:row>
     <x:row r="173" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A173" s="99" t="n">
-        <x:v>172</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B173" s="20" t="str">
         <x:v>Tai Felton</x:v>
@@ -17758,7 +17761,7 @@
     </x:row>
     <x:row r="174" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A174" s="99" t="n">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B174" s="20" t="str">
         <x:v>CJ Daniels</x:v>
@@ -17802,7 +17805,7 @@
     </x:row>
     <x:row r="175" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A175" s="99" t="n">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B175" s="20" t="str">
         <x:v>Isaiah Williams</x:v>
@@ -17934,7 +17937,7 @@
     </x:row>
     <x:row r="178" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A178" s="99" t="n">
-        <x:v>177</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B178" s="20" t="str">
         <x:v>Tyrell Shavers</x:v>
@@ -17978,7 +17981,7 @@
     </x:row>
     <x:row r="179" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A179" s="99" t="n">
-        <x:v>178</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="B179" s="20" t="str">
         <x:v>Cody White</x:v>
@@ -18022,7 +18025,7 @@
     </x:row>
     <x:row r="180" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A180" s="99" t="n">
-        <x:v>179</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B180" s="20" t="str">
         <x:v>Malachi Corley</x:v>
@@ -18110,7 +18113,7 @@
     </x:row>
     <x:row r="182" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A182" s="99" t="n">
-        <x:v>181</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B182" s="20" t="str">
         <x:v>Mason Tipton</x:v>
@@ -18154,7 +18157,7 @@
     </x:row>
     <x:row r="183" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A183" s="99" t="n">
-        <x:v>182</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B183" s="20" t="str">
         <x:v>David Moore</x:v>
@@ -18198,7 +18201,7 @@
     </x:row>
     <x:row r="184" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A184" s="99" t="n">
-        <x:v>183</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="B184" s="20" t="str">
         <x:v>Jonathan Mingo</x:v>
@@ -18242,7 +18245,7 @@
     </x:row>
     <x:row r="185" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A185" s="99" t="n">
-        <x:v>184</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B185" s="20" t="str">
         <x:v>Chase Roberts</x:v>
@@ -18286,7 +18289,7 @@
     </x:row>
     <x:row r="186" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A186" s="99" t="n">
-        <x:v>185</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B186" s="20" t="str">
         <x:v>Kaden Wetjen</x:v>
@@ -18330,7 +18333,7 @@
     </x:row>
     <x:row r="187" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A187" s="99" t="n">
-        <x:v>186</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B187" s="20" t="str">
         <x:v>Anthony Gould</x:v>
@@ -18418,7 +18421,7 @@
     </x:row>
     <x:row r="189" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A189" s="99" t="n">
-        <x:v>188</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="B189" s="20" t="str">
         <x:v>Tyler Johnson</x:v>
@@ -18462,7 +18465,7 @@
     </x:row>
     <x:row r="190" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A190" s="99" t="n">
-        <x:v>189</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B190" s="20" t="str">
         <x:v>Justin Watson</x:v>
@@ -18506,7 +18509,7 @@
     </x:row>
     <x:row r="191" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A191" s="99" t="n">
-        <x:v>190</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B191" s="20" t="str">
         <x:v>Jake Bobo</x:v>
@@ -18726,7 +18729,7 @@
     </x:row>
     <x:row r="196" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A196" s="99" t="n">
-        <x:v>195</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B196" s="20" t="str">
         <x:v>Arian Smith</x:v>
@@ -18770,7 +18773,7 @@
     </x:row>
     <x:row r="197" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A197" s="99" t="n">
-        <x:v>196</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B197" s="20" t="str">
         <x:v>Chris Moore</x:v>
@@ -18814,7 +18817,7 @@
     </x:row>
     <x:row r="198" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A198" s="99" t="n">
-        <x:v>197</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B198" s="20" t="str">
         <x:v>Ricky White III</x:v>
@@ -18902,7 +18905,7 @@
     </x:row>
     <x:row r="200" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A200" s="99" t="n">
-        <x:v>199</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B200" s="20" t="str">
         <x:v>Emmanuel Henderson Jr.</x:v>
@@ -18946,7 +18949,7 @@
     </x:row>
     <x:row r="201" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A201" s="99" t="n">
-        <x:v>200</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="B201" s="20" t="str">
         <x:v>Bryce Oliver</x:v>
@@ -18990,7 +18993,7 @@
     </x:row>
     <x:row r="202" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A202" s="99" t="n">
-        <x:v>201</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B202" s="20" t="str">
         <x:v>Jordan Watkins</x:v>
@@ -19034,7 +19037,7 @@
     </x:row>
     <x:row r="203" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A203" s="99" t="n">
-        <x:v>202</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B203" s="20" t="str">
         <x:v>Kameron Johnson</x:v>
@@ -19078,7 +19081,7 @@
     </x:row>
     <x:row r="204" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A204" s="99" t="n">
-        <x:v>203</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B204" s="20" t="str">
         <x:v>JuJu Smith-Schuster</x:v>
@@ -19122,7 +19125,7 @@
     </x:row>
     <x:row r="205" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A205" s="99" t="n">
-        <x:v>204</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B205" s="20" t="str">
         <x:v>Jayden Higgins</x:v>
@@ -19166,7 +19169,7 @@
     </x:row>
     <x:row r="206" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A206" s="99" t="n">
-        <x:v>205</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B206" s="20" t="str">
         <x:v>A.T. Perry</x:v>
@@ -19210,7 +19213,7 @@
     </x:row>
     <x:row r="207" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A207" s="99" t="n">
-        <x:v>206</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B207" s="20" t="str">
         <x:v>Anthony Smith</x:v>
@@ -19254,7 +19257,7 @@
     </x:row>
     <x:row r="208" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A208" s="99" t="n">
-        <x:v>207</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B208" s="20" t="str">
         <x:v>Braxton Berrios</x:v>
@@ -19298,7 +19301,7 @@
     </x:row>
     <x:row r="209" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A209" s="99" t="n">
-        <x:v>208</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="B209" s="20" t="str">
         <x:v>Britain Covey</x:v>
@@ -19342,7 +19345,7 @@
     </x:row>
     <x:row r="210" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A210" s="99" t="n">
-        <x:v>209</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B210" s="20" t="str">
         <x:v>Casey Washington</x:v>
@@ -19386,7 +19389,7 @@
     </x:row>
     <x:row r="211" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A211" s="99" t="n">
-        <x:v>210</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="B211" s="20" t="str">
         <x:v>Cedrick Wilson Jr.</x:v>
@@ -19430,7 +19433,7 @@
     </x:row>
     <x:row r="212" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A212" s="99" t="n">
-        <x:v>211</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="B212" s="20" t="str">
         <x:v>Charlie Jones</x:v>
@@ -19474,7 +19477,7 @@
     </x:row>
     <x:row r="213" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A213" s="99" t="n">
-        <x:v>212</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="B213" s="20" t="str">
         <x:v>Chris Brazzell II</x:v>
@@ -19518,7 +19521,7 @@
     </x:row>
     <x:row r="214" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A214" s="99" t="n">
-        <x:v>213</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="B214" s="20" t="str">
         <x:v>Danny Gray</x:v>
@@ -19562,7 +19565,7 @@
     </x:row>
     <x:row r="215" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A215" s="99" t="n">
-        <x:v>214</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="B215" s="20" t="str">
         <x:v>Dante Pettis</x:v>
@@ -19606,7 +19609,7 @@
     </x:row>
     <x:row r="216" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A216" s="99" t="n">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B216" s="20" t="str">
         <x:v>Dareke Young</x:v>
@@ -19650,7 +19653,7 @@
     </x:row>
     <x:row r="217" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A217" s="99" t="n">
-        <x:v>216</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="B217" s="20" t="str">
         <x:v>Deven Thompkins</x:v>
@@ -19694,7 +19697,7 @@
     </x:row>
     <x:row r="218" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A218" s="99" t="n">
-        <x:v>217</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B218" s="20" t="str">
         <x:v>Devin Duvernay</x:v>
@@ -19738,7 +19741,7 @@
     </x:row>
     <x:row r="219" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A219" s="99" t="n">
-        <x:v>218</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B219" s="20" t="str">
         <x:v>Dominic Lovett</x:v>
@@ -19782,7 +19785,7 @@
     </x:row>
     <x:row r="220" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A220" s="99" t="n">
-        <x:v>219</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="B220" s="20" t="str">
         <x:v>Efton Chism III</x:v>
@@ -19826,7 +19829,7 @@
     </x:row>
     <x:row r="221" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A221" s="99" t="n">
-        <x:v>220</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="B221" s="20" t="str">
         <x:v>Gage Larvadain</x:v>
@@ -19870,7 +19873,7 @@
     </x:row>
     <x:row r="222" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A222" s="99" t="n">
-        <x:v>221</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B222" s="20" t="str">
         <x:v>Gunner Olszewski</x:v>
@@ -19914,7 +19917,7 @@
     </x:row>
     <x:row r="223" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A223" s="99" t="n">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="B223" s="20" t="str">
         <x:v>Ihmir Smith-Marsette</x:v>
@@ -19958,7 +19961,7 @@
     </x:row>
     <x:row r="224" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A224" s="99" t="n">
-        <x:v>223</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B224" s="20" t="str">
         <x:v>Irv Charles</x:v>
@@ -20002,7 +20005,7 @@
     </x:row>
     <x:row r="225" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A225" s="99" t="n">
-        <x:v>224</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B225" s="20" t="str">
         <x:v>Isaiah Neyor</x:v>
@@ -20046,7 +20049,7 @@
     </x:row>
     <x:row r="226" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A226" s="99" t="n">
-        <x:v>225</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="B226" s="20" t="str">
         <x:v>Jacob Cowing</x:v>
@@ -20090,7 +20093,7 @@
     </x:row>
     <x:row r="227" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A227" s="99" t="n">
-        <x:v>226</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B227" s="20" t="str">
         <x:v>Jalen Brooks</x:v>
@@ -20134,7 +20137,7 @@
     </x:row>
     <x:row r="228" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A228" s="99" t="n">
-        <x:v>227</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="B228" s="20" t="str">
         <x:v>Jalin Hyatt</x:v>
@@ -20178,7 +20181,7 @@
     </x:row>
     <x:row r="229" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A229" s="99" t="n">
-        <x:v>228</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="B229" s="20" t="str">
         <x:v>Jamari Thrash</x:v>
@@ -20222,7 +20225,7 @@
     </x:row>
     <x:row r="230" s="42" customFormat="1" ht="15" customHeight="1">
       <x:c r="A230" s="99" t="n">
-        <x:v>229</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="B230" s="20" t="str">
         <x:v>Jason Brownlee</x:v>
@@ -21411,7 +21414,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0c708d7afd24196"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6636e7ee4f8e42ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28331,7 +28334,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37bd1d8da4af4175"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1e10696af80409d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28375,7 +28378,7 @@
         <x:v>Updated</x:v>
       </x:c>
       <x:c r="B2" s="46" t="str">
-        <x:v>August 24, 2026, 10:46 AM ET</x:v>
+        <x:v>August 30, 2026, 12:00 PM ET</x:v>
       </x:c>
       <x:c r="C2" s="46" t="str">
         <x:v>Timezone</x:v>
@@ -32886,6 +32889,120 @@
       <x:c r="K132"/>
       <x:c r="L132"/>
     </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>Kayshon Boutte</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>HOU</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>TEAM UPDATED</x:v>
+      </x:c>
+      <x:c r="E133" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="F133" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="G133" t="n">
+        <x:v>73.9</x:v>
+      </x:c>
+      <x:c r="H133" t="n">
+        <x:v>73.9</x:v>
+      </x:c>
+      <x:c r="I133" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J133" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K133" t="str">
+        <x:v>Team updated after Houston officially acquired Boutte from New England; workload projection is unchanged pending role evidence.</x:v>
+      </x:c>
+      <x:c r="L133" t="str">
+        <x:v>https://www.houstontexans.com/news/houston-texans-transactions-8-25-2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>Tutu Atwell</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>LAR</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>TEAM UPDATED</x:v>
+      </x:c>
+      <x:c r="E134" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F134" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="G134" t="n">
+        <x:v>33.9</x:v>
+      </x:c>
+      <x:c r="H134" t="n">
+        <x:v>33.9</x:v>
+      </x:c>
+      <x:c r="I134" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J134" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K134" t="str">
+        <x:v>Team updated after the Rams officially reacquired Atwell from Miami; workload projection is unchanged pending role evidence.</x:v>
+      </x:c>
+      <x:c r="L134" t="str">
+        <x:v>https://www.therams.com/news/rams-agree-to-trade-rb-jarquez-hunter-to-dolphins-for-wr-tutu-atwell</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>WR</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>Cedric Tillman</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>FA</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>REMOVED FROM ACTIVE PROJECTION</x:v>
+      </x:c>
+      <x:c r="E135" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="F135" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="G135" t="n">
+        <x:v>68.8</x:v>
+      </x:c>
+      <x:c r="H135" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I135" t="n">
+        <x:v>-68.8</x:v>
+      </x:c>
+      <x:c r="J135" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K135" t="str">
+        <x:v>Cleveland waived Tillman, so his active-team workload is removed until he signs elsewhere and a new role is established.</x:v>
+      </x:c>
+      <x:c r="L135" t="str">
+        <x:v>https://x.com/DanielOyefusi/status/2093081141716660460</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A54:L54"/>

</xml_diff>